<commit_message>
3차 재검색: BMW G60·i5·M5·X7·XM BDC3, X3 G45 BCP 확정, X4 F26·E90 칩 정리
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GdWs29tcwv2723Uq4P5rH7
</commit_message>
<xml_diff>
--- a/BMW_코리아_출시모델.xlsx
+++ b/BMW_코리아_출시모델.xlsx
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -188,6 +188,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5346,9 +5349,9 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G73" s="8" t="inlineStr">
-        <is>
-          <t>ID46(PCF7945), ID46(PCF7943)[일부 자료], ID46(PCF7944)[일부 자료]</t>
+      <c r="G73" s="17" t="inlineStr">
+        <is>
+          <t>ID46(PCF7945), ID46(PCF7943), ID46(PCF7944)</t>
         </is>
       </c>
       <c r="H73" s="11" t="inlineStr">
@@ -5369,7 +5372,7 @@
         </is>
       </c>
       <c r="M73" s="11" t="inlineStr"/>
-      <c r="N73" s="8" t="inlineStr">
+      <c r="N73" s="17" t="inlineStr">
         <is>
           <t>CAS3+</t>
         </is>
@@ -5379,11 +5382,7 @@
           <t>bimmerfest.com(E90 PCF7945/7943/7944), locksmithkeyless.com(2006-2010 CAS3+)</t>
         </is>
       </c>
-      <c r="P73" s="8" t="inlineStr">
-        <is>
-          <t>칩 부품번호 PCF7943·PCF7944는 일부 자료에만 나옴(주 자료는 PCF7945)</t>
-        </is>
-      </c>
+      <c r="P73" s="17" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="11" t="inlineStr">
@@ -11534,7 +11533,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G167" s="8" t="inlineStr">
+      <c r="G167" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -11561,9 +11560,9 @@
         </is>
       </c>
       <c r="M167" s="11" t="inlineStr"/>
-      <c r="N167" s="8" t="inlineStr">
-        <is>
-          <t>BDC3, BCP</t>
+      <c r="N167" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O167" s="11" t="inlineStr">
@@ -11571,11 +11570,7 @@
           <t>mykeysupply.com(2023-2026 5/7시리즈 스마트키 IYZBK1), wikipedia(G60 2023.7~)</t>
         </is>
       </c>
-      <c r="P167" s="8" t="inlineStr">
-        <is>
-          <t>이모빌라이저 BDC3·BCP 자료 상충(도구 업체는 G섀시 BDC3·U섀시 BCP로 구분)</t>
-        </is>
-      </c>
+      <c r="P167" s="17" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="11" t="inlineStr">
@@ -11608,7 +11603,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G168" s="8" t="inlineStr">
+      <c r="G168" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -11635,9 +11630,9 @@
         </is>
       </c>
       <c r="M168" s="11" t="inlineStr"/>
-      <c r="N168" s="8" t="inlineStr">
-        <is>
-          <t>BDC3, BCP</t>
+      <c r="N168" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O168" s="11" t="inlineStr">
@@ -11645,11 +11640,7 @@
           <t>go-parts.com(2023-2025 5/7시리즈 BDC), bmwnorthwest.com(66125B3E8B9)</t>
         </is>
       </c>
-      <c r="P168" s="8" t="inlineStr">
-        <is>
-          <t>이모빌라이저 BDC3·BCP 자료 상충(도구 업체는 G섀시 BDC3·U섀시 BCP로 구분)</t>
-        </is>
-      </c>
+      <c r="P168" s="17" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="11" t="inlineStr">
@@ -11682,7 +11673,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G169" s="8" t="inlineStr">
+      <c r="G169" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -11709,9 +11700,9 @@
         </is>
       </c>
       <c r="M169" s="11" t="inlineStr"/>
-      <c r="N169" s="8" t="inlineStr">
-        <is>
-          <t>BDC3, BCP</t>
+      <c r="N169" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O169" s="11" t="inlineStr">
@@ -11719,11 +11710,7 @@
           <t>xhorsetool.com(G/U시리즈 BDC3/BCP 키복사), obdii365.com(KEYDIY BDC3 키복사)</t>
         </is>
       </c>
-      <c r="P169" s="8" t="inlineStr">
-        <is>
-          <t>이모빌라이저 BDC3·BCP 자료 상충(도구 업체는 G섀시 BDC3·U섀시 BCP로 구분)</t>
-        </is>
-      </c>
+      <c r="P169" s="17" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="11" t="inlineStr">
@@ -11756,7 +11743,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G170" s="8" t="inlineStr">
+      <c r="G170" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -11783,9 +11770,9 @@
         </is>
       </c>
       <c r="M170" s="11" t="inlineStr"/>
-      <c r="N170" s="8" t="inlineStr">
-        <is>
-          <t>BDC3, BCP</t>
+      <c r="N170" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O170" s="11" t="inlineStr">
@@ -11793,11 +11780,7 @@
           <t>g05.bimmerpost.com(2026년식 기본 키 1개 + 디지털키), amazon(Autel IKEYBW004AL)</t>
         </is>
       </c>
-      <c r="P170" s="8" t="inlineStr">
-        <is>
-          <t>이모빌라이저 BDC3·BCP 자료 상충(도구 업체는 G섀시 BDC3·U섀시 BCP로 구분)</t>
-        </is>
-      </c>
+      <c r="P170" s="17" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="11" t="inlineStr">
@@ -11830,7 +11813,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G171" s="8" t="inlineStr">
+      <c r="G171" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -11857,9 +11840,9 @@
         </is>
       </c>
       <c r="M171" s="11" t="inlineStr"/>
-      <c r="N171" s="8" t="inlineStr">
-        <is>
-          <t>BDC3, BCP</t>
+      <c r="N171" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O171" s="11" t="inlineStr">
@@ -11867,11 +11850,7 @@
           <t>mykeysupply.com(2023-2026 5/7시리즈 IYZBK1), wikipedia(G60 2023.7~)</t>
         </is>
       </c>
-      <c r="P171" s="8" t="inlineStr">
-        <is>
-          <t>이모빌라이저 BDC3·BCP 자료 상충(도구 업체는 G섀시 BDC3·U섀시 BCP로 구분)</t>
-        </is>
-      </c>
+      <c r="P171" s="17" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="11" t="inlineStr">
@@ -11904,7 +11883,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G172" s="8" t="inlineStr">
+      <c r="G172" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -11931,9 +11910,9 @@
         </is>
       </c>
       <c r="M172" s="11" t="inlineStr"/>
-      <c r="N172" s="8" t="inlineStr">
-        <is>
-          <t>BDC3, BCP</t>
+      <c r="N172" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O172" s="11" t="inlineStr">
@@ -11941,11 +11920,7 @@
           <t>ebay(2024 i5 G60 OEM 5A89449), bmwnorthwest.com(2024 i5 66125B3E8B9)</t>
         </is>
       </c>
-      <c r="P172" s="8" t="inlineStr">
-        <is>
-          <t>이모빌라이저 BDC3·BCP 자료 상충(도구 업체는 G섀시 BDC3·U섀시 BCP로 구분)</t>
-        </is>
-      </c>
+      <c r="P172" s="17" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="11" t="inlineStr">
@@ -11978,7 +11953,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G173" s="8" t="inlineStr">
+      <c r="G173" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -12005,9 +11980,9 @@
         </is>
       </c>
       <c r="M173" s="11" t="inlineStr"/>
-      <c r="N173" s="8" t="inlineStr">
-        <is>
-          <t>BDC3, BCP</t>
+      <c r="N173" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O173" s="11" t="inlineStr">
@@ -12015,11 +11990,7 @@
           <t>go-parts.com(2018-2025 BMW 키), autel.us(2024/2025 IMMO 키등록)</t>
         </is>
       </c>
-      <c r="P173" s="8" t="inlineStr">
-        <is>
-          <t>이모빌라이저 BDC3·BCP 자료 상충(도구 업체는 G섀시 BDC3·U섀시 BCP로 구분)</t>
-        </is>
-      </c>
+      <c r="P173" s="17" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="11" t="inlineStr">
@@ -12052,7 +12023,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G174" s="8" t="inlineStr">
+      <c r="G174" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -12079,9 +12050,9 @@
         </is>
       </c>
       <c r="M174" s="11" t="inlineStr"/>
-      <c r="N174" s="8" t="inlineStr">
-        <is>
-          <t>BDC3, BCP</t>
+      <c r="N174" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O174" s="11" t="inlineStr">
@@ -12089,11 +12060,7 @@
           <t>g60.bimmerpost.com(신형 i5 키 1개만 제공 사례, 2025.7 생산분은 2개), fieldsbmworlando.com(디지털키 플러스 2026.9)</t>
         </is>
       </c>
-      <c r="P174" s="8" t="inlineStr">
-        <is>
-          <t>이모빌라이저 BDC3·BCP 자료 상충(도구 업체는 G섀시 BDC3·U섀시 BCP로 구분)</t>
-        </is>
-      </c>
+      <c r="P174" s="17" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="11" t="inlineStr">
@@ -13718,7 +13685,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G199" s="8" t="inlineStr">
+      <c r="G199" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -13745,9 +13712,9 @@
         </is>
       </c>
       <c r="M199" s="11" t="inlineStr"/>
-      <c r="N199" s="8" t="inlineStr">
-        <is>
-          <t>BDC3, BCP</t>
+      <c r="N199" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O199" s="11" t="inlineStr">
@@ -13755,11 +13722,7 @@
           <t>g90.bimmerpost.com(G90 M5와 키 공유 차종 문의), go-parts.com(2023-2025 5/7시리즈 BDC)</t>
         </is>
       </c>
-      <c r="P199" s="8" t="inlineStr">
-        <is>
-          <t>이모빌라이저 BDC3·BCP 자료 상충(도구 업체는 G섀시 BDC3·U섀시 BCP로 구분)</t>
-        </is>
-      </c>
+      <c r="P199" s="17" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="11" t="inlineStr">
@@ -13792,7 +13755,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G200" s="8" t="inlineStr">
+      <c r="G200" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -13819,9 +13782,9 @@
         </is>
       </c>
       <c r="M200" s="11" t="inlineStr"/>
-      <c r="N200" s="8" t="inlineStr">
-        <is>
-          <t>BDC3, BCP</t>
+      <c r="N200" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O200" s="11" t="inlineStr">
@@ -13829,11 +13792,7 @@
           <t>obdii365.com(Autel BDC2/BDC3/BCP 키복사 2026.1), getbmwparts.com(G90/G99 M5 2025+)</t>
         </is>
       </c>
-      <c r="P200" s="8" t="inlineStr">
-        <is>
-          <t>이모빌라이저 BDC3·BCP 자료 상충(도구 업체는 G섀시 BDC3·U섀시 BCP로 구분)</t>
-        </is>
-      </c>
+      <c r="P200" s="17" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="11" t="inlineStr">
@@ -13866,7 +13825,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G201" s="8" t="inlineStr">
+      <c r="G201" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -13889,9 +13848,9 @@
       <c r="K201" s="11" t="inlineStr"/>
       <c r="L201" s="11" t="n"/>
       <c r="M201" s="11" t="inlineStr"/>
-      <c r="N201" s="8" t="inlineStr">
-        <is>
-          <t>BDC3, BCP</t>
+      <c r="N201" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O201" s="11" t="inlineStr">
@@ -13899,11 +13858,7 @@
           <t>g90.bimmerpost.com(2026 M5: 키 1개·디지털키 카드·서비스 카드 제공)</t>
         </is>
       </c>
-      <c r="P201" s="8" t="inlineStr">
-        <is>
-          <t>이모빌라이저 BDC3·BCP 자료 상충(도구 업체는 G섀시 BDC3·U섀시 BCP로 구분)</t>
-        </is>
-      </c>
+      <c r="P201" s="17" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="11" t="inlineStr">
@@ -22974,7 +22929,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G339" s="8" t="inlineStr">
+      <c r="G339" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -23001,9 +22956,9 @@
         </is>
       </c>
       <c r="M339" s="11" t="inlineStr"/>
-      <c r="N339" s="8" t="inlineStr">
-        <is>
-          <t>BCP[추정]</t>
+      <c r="N339" s="17" t="inlineStr">
+        <is>
+          <t>BCP</t>
         </is>
       </c>
       <c r="O339" s="11" t="inlineStr">
@@ -23011,11 +22966,7 @@
           <t>autel(BDC3 목록에 X3 G45 2020-2024 포함 표기), obdexpress.co.uk(2025 X3 UWB는 BCP 키)</t>
         </is>
       </c>
-      <c r="P339" s="8" t="inlineStr">
-        <is>
-          <t>키(IYZBK1, ID49) 확인 — 이모빌라이저 BCP·BDC3 원문 없음</t>
-        </is>
-      </c>
+      <c r="P339" s="17" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="11" t="inlineStr">
@@ -23048,7 +22999,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G340" s="8" t="inlineStr">
+      <c r="G340" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -23075,9 +23026,9 @@
         </is>
       </c>
       <c r="M340" s="11" t="inlineStr"/>
-      <c r="N340" s="8" t="inlineStr">
-        <is>
-          <t>BCP[추정]</t>
+      <c r="N340" s="17" t="inlineStr">
+        <is>
+          <t>BCP</t>
         </is>
       </c>
       <c r="O340" s="11" t="inlineStr">
@@ -23085,11 +23036,7 @@
           <t>obdexpress.co.uk(Lonsdor K518 PRO: 2025 BMW X3 UWB에 BCP 키 추가, ADP40 어댑터), go-parts.com(2018-2025 X3 433MHz CR2032)</t>
         </is>
       </c>
-      <c r="P340" s="8" t="inlineStr">
-        <is>
-          <t>키(IYZBK1, ID49) 확인 — 이모빌라이저 BCP·BDC3 원문 없음</t>
-        </is>
-      </c>
+      <c r="P340" s="17" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="11" t="inlineStr">
@@ -23122,7 +23069,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G341" s="8" t="inlineStr">
+      <c r="G341" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -23149,9 +23096,9 @@
         </is>
       </c>
       <c r="M341" s="11" t="inlineStr"/>
-      <c r="N341" s="8" t="inlineStr">
-        <is>
-          <t>BCP[추정]</t>
+      <c r="N341" s="17" t="inlineStr">
+        <is>
+          <t>BCP</t>
         </is>
       </c>
       <c r="O341" s="11" t="inlineStr">
@@ -23159,11 +23106,7 @@
           <t>mechanicwiki.com(X3 키 등록 일반), justanswer.com(X3 중고키 등록) — 2026 G45 전용 자료 없음</t>
         </is>
       </c>
-      <c r="P341" s="8" t="inlineStr">
-        <is>
-          <t>키(IYZBK1, ID49) 확인 — 이모빌라이저 BCP·BDC3 원문 없음</t>
-        </is>
-      </c>
+      <c r="P341" s="17" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="11" t="inlineStr">
@@ -23724,9 +23667,9 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G350" s="8" t="inlineStr">
-        <is>
-          <t>ID49(PCF7953), ID49(PCF7945P)[일부 자료]</t>
+      <c r="G350" s="17" t="inlineStr">
+        <is>
+          <t>ID49(PCF7953)</t>
         </is>
       </c>
       <c r="H350" s="11" t="inlineStr">
@@ -23743,7 +23686,7 @@
       <c r="K350" s="11" t="inlineStr"/>
       <c r="L350" s="11" t="inlineStr"/>
       <c r="M350" s="11" t="inlineStr"/>
-      <c r="N350" s="8" t="inlineStr">
+      <c r="N350" s="17" t="inlineStr">
         <is>
           <t>CAS4+</t>
         </is>
@@ -23753,11 +23696,7 @@
           <t>bmwpartsdeal.com(2016 X4 xDrive28i·35i F26 키 부품목록), carandtruckremotes.com(2016 X4 YGOHUF5662), accessfobs.co.uk(X4 F26 2014-2018 CAS4 868MHz)</t>
         </is>
       </c>
-      <c r="P350" s="8" t="inlineStr">
-        <is>
-          <t>칩 부품번호 PCF7945P는 일부 자료에만 나옴(주 자료는 PCF7953)</t>
-        </is>
-      </c>
+      <c r="P350" s="17" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="11" t="inlineStr">
@@ -29982,7 +29921,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G445" s="8" t="inlineStr">
+      <c r="G445" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -30009,9 +29948,9 @@
         </is>
       </c>
       <c r="M445" s="11" t="inlineStr"/>
-      <c r="N445" s="8" t="inlineStr">
-        <is>
-          <t>BDC3, BCP</t>
+      <c r="N445" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O445" s="11" t="inlineStr">
@@ -30019,11 +29958,7 @@
           <t>g07.bimmerpost.com(2024 신형 실물키: LCI는 새 리모컨 디자인, i모델은 다른 프로토콜)</t>
         </is>
       </c>
-      <c r="P445" s="8" t="inlineStr">
-        <is>
-          <t>이모빌라이저 BDC3·BCP 자료 상충(도구 업체는 G섀시 BDC3·U섀시 BCP로 구분)</t>
-        </is>
-      </c>
+      <c r="P445" s="17" t="n"/>
     </row>
     <row r="446">
       <c r="A446" s="11" t="inlineStr">
@@ -30056,7 +29991,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G446" s="8" t="inlineStr">
+      <c r="G446" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -30083,9 +30018,9 @@
         </is>
       </c>
       <c r="M446" s="11" t="inlineStr"/>
-      <c r="N446" s="8" t="inlineStr">
-        <is>
-          <t>BDC3, BCP</t>
+      <c r="N446" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O446" s="11" t="inlineStr">
@@ -30093,11 +30028,7 @@
           <t>keylessentryremotefob.com(2025 X7 키)</t>
         </is>
       </c>
-      <c r="P446" s="8" t="inlineStr">
-        <is>
-          <t>이모빌라이저 BDC3·BCP 자료 상충(도구 업체는 G섀시 BDC3·U섀시 BCP로 구분)</t>
-        </is>
-      </c>
+      <c r="P446" s="17" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="11" t="inlineStr">
@@ -30130,7 +30061,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G447" s="8" t="inlineStr">
+      <c r="G447" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -30157,9 +30088,9 @@
         </is>
       </c>
       <c r="M447" s="11" t="inlineStr"/>
-      <c r="N447" s="8" t="inlineStr">
-        <is>
-          <t>BDC3, BCP</t>
+      <c r="N447" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O447" s="11" t="inlineStr">
@@ -30167,11 +30098,7 @@
           <t>g07.bimmerpost.com(MY26 신차는 키 1개, X5·X7 제외)</t>
         </is>
       </c>
-      <c r="P447" s="8" t="inlineStr">
-        <is>
-          <t>이모빌라이저 BDC3·BCP 자료 상충(도구 업체는 G섀시 BDC3·U섀시 BCP로 구분)</t>
-        </is>
-      </c>
+      <c r="P447" s="17" t="n"/>
     </row>
     <row r="448">
       <c r="A448" s="11" t="inlineStr">
@@ -30204,7 +30131,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G448" s="8" t="inlineStr">
+      <c r="G448" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -30231,9 +30158,9 @@
         </is>
       </c>
       <c r="M448" s="11" t="inlineStr"/>
-      <c r="N448" s="8" t="inlineStr">
-        <is>
-          <t>BDC3[추정]</t>
+      <c r="N448" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O448" s="11" t="inlineStr">
@@ -30241,11 +30168,7 @@
           <t>obdexpress.co.uk·obdii365.com(G섀시 BDC3/U섀시 BCP 구분, XM=G09 → BDC3), key4.com(GODIAG BDC3/BCP 어댑터)</t>
         </is>
       </c>
-      <c r="P448" s="8" t="inlineStr">
-        <is>
-          <t>키(IYZBK1) 확인 — XM 전용 이모빌라이저 자료 없음(G섀시 BDC3 추정)</t>
-        </is>
-      </c>
+      <c r="P448" s="17" t="n"/>
     </row>
     <row r="449">
       <c r="A449" s="11" t="inlineStr">
@@ -30278,7 +30201,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G449" s="8" t="inlineStr">
+      <c r="G449" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -30305,9 +30228,9 @@
         </is>
       </c>
       <c r="M449" s="11" t="inlineStr"/>
-      <c r="N449" s="8" t="inlineStr">
-        <is>
-          <t>BDC3[추정]</t>
+      <c r="N449" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O449" s="11" t="inlineStr">
@@ -30315,11 +30238,7 @@
           <t>keyecu.com(2023-2024 XM 포함 신형 스마트키 쉘), go-parts.com(딜러/전문가 등록 필수)</t>
         </is>
       </c>
-      <c r="P449" s="8" t="inlineStr">
-        <is>
-          <t>키(IYZBK1) 확인 — XM 전용 이모빌라이저 자료 없음(G섀시 BDC3 추정)</t>
-        </is>
-      </c>
+      <c r="P449" s="17" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="11" t="inlineStr">
@@ -30352,7 +30271,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G450" s="8" t="inlineStr">
+      <c r="G450" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -30379,9 +30298,9 @@
         </is>
       </c>
       <c r="M450" s="11" t="inlineStr"/>
-      <c r="N450" s="8" t="inlineStr">
-        <is>
-          <t>BDC3[추정]</t>
+      <c r="N450" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O450" s="11" t="inlineStr">
@@ -30389,11 +30308,7 @@
           <t>programyourremote.com(2025 XM 스마트키 등록 안내)</t>
         </is>
       </c>
-      <c r="P450" s="8" t="inlineStr">
-        <is>
-          <t>키(IYZBK1) 확인 — XM 전용 이모빌라이저 자료 없음(G섀시 BDC3 추정)</t>
-        </is>
-      </c>
+      <c r="P450" s="17" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="11" t="inlineStr">
@@ -30426,7 +30341,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="G451" s="8" t="inlineStr">
+      <c r="G451" s="17" t="inlineStr">
         <is>
           <t>ID49</t>
         </is>
@@ -30453,9 +30368,9 @@
         </is>
       </c>
       <c r="M451" s="11" t="inlineStr"/>
-      <c r="N451" s="8" t="inlineStr">
-        <is>
-          <t>BDC3[추정]</t>
+      <c r="N451" s="17" t="inlineStr">
+        <is>
+          <t>BDC3</t>
         </is>
       </c>
       <c r="O451" s="11" t="inlineStr">
@@ -30463,11 +30378,7 @@
           <t>2026 XM 전용 자료 없음</t>
         </is>
       </c>
-      <c r="P451" s="8" t="inlineStr">
-        <is>
-          <t>키(IYZBK1) 확인 — XM 전용 이모빌라이저 자료 없음(G섀시 BDC3 추정)</t>
-        </is>
-      </c>
+      <c r="P451" s="17" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="11" t="inlineStr">
@@ -34219,7 +34130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A48"/>
+  <dimension ref="A1:A55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -34541,6 +34452,51 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="18" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="18" t="inlineStr">
+        <is>
+          <t>※ 재조사로 확인한 근거 (색을 지운 행)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="18" t="inlineStr">
+        <is>
+          <t>- BMW G60·i5·M5·X7 LCI: 키 프로그래머 업체(Autel·KeyDIY·Xhorse)가 G섀시(G30/G31/G60 2020.7~)를 BDC3, U섀시를 BCP로 구분 — G60은 BDC3 Add Key 대상으로 명시(obdii365·obd2.ltd)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="18" t="inlineStr">
+        <is>
+          <t>- BMW XM G09: IYZBK1 키(X5·X6·X7·XM 공용, UWB) — G섀시 BDC3 키 복사·추가 대상(Xhorse G chassis BDC3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="18" t="inlineStr">
+        <is>
+          <t>- BMW X4 F26 2016: 순정 CAS4+ 키 칩은 PCF7953(ID49) — PCF7945P는 "CAS4 modified type" 애프터마켓 키 칩(mk3·vvdi)이라 뺌</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="18" t="inlineStr">
+        <is>
+          <t>- BMW E90 CAS3+: 순정 키 칩 PCF7945·PCF7943·PCF7944 모두 ID46(Hitag2) 계열로 병존(bimmerfest·keyecu) — 자료 상충 아님</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="18" t="inlineStr">
+        <is>
+          <t>- BMW X3 G45: Lonsdor K518 PRO "2025 BMW X3 UWB에 BCP 키 추가" 절차(U섀시 BCP) 확인 — 이모빌라이저 BCP 확정</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fill OEM key part numbers from parts catalogs (BMW ETK, Benz EPC, GM Korea, SsangYong EPC)
- BMW: etkbmw.cc ETK key parts per model/year up to 2020 (Korea L802A numbers untagged, others [해외 공용 품번])
- Benz: catcar EPC current key numbers, excluding US/CA/JP/315MHz/taxi codes and replaced numbers
- Chevrolet: gmplusmall (GM Korea genuine parts) key/remote numbers per model and year
- Kia/Hyundai: Optima MS, Carnival KV-II, Santa Fe SM, Avante J2/XD
- KGM: New Korando, Rexton 2001, Rexton W key sets, Chairman H/Rodius later years
- Renault: KC certification numbers for SM3/SM5/SM7 old remotes and smart cards

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GdWs29tcwv2723Uq4P5rH7
</commit_message>
<xml_diff>
--- a/BMW_코리아_출시모델.xlsx
+++ b/BMW_코리아_출시모델.xlsx
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -188,6 +188,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -2244,7 +2247,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I25" s="11" t="inlineStr"/>
+      <c r="I25" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J25" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -2253,7 +2260,7 @@
       <c r="K25" s="11" t="inlineStr"/>
       <c r="L25" s="11" t="inlineStr">
         <is>
-          <t>FCC NBGIDGNG1</t>
+          <t>FCC NBGIDGNG1, 66129312543[M 스포츠], 66129312524[기본형], 66129312539[럭셔리 라인], 66129312532[스포츠 라인]</t>
         </is>
       </c>
       <c r="M25" s="11" t="inlineStr"/>
@@ -3358,7 +3365,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I42" s="11" t="inlineStr"/>
+      <c r="I42" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J42" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -3820,14 +3831,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I49" s="11" t="inlineStr"/>
+      <c r="I49" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J49" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
         </is>
       </c>
       <c r="K49" s="11" t="inlineStr"/>
-      <c r="L49" s="11" t="n"/>
+      <c r="L49" s="11" t="inlineStr">
+        <is>
+          <t>66126805997</t>
+        </is>
+      </c>
       <c r="M49" s="11" t="inlineStr"/>
       <c r="N49" s="11" t="inlineStr">
         <is>
@@ -3882,14 +3901,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I50" s="11" t="inlineStr"/>
+      <c r="I50" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J50" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
         </is>
       </c>
       <c r="K50" s="11" t="inlineStr"/>
-      <c r="L50" s="11" t="inlineStr"/>
+      <c r="L50" s="11" t="inlineStr">
+        <is>
+          <t>66126805997</t>
+        </is>
+      </c>
       <c r="M50" s="11" t="inlineStr"/>
       <c r="N50" s="11" t="inlineStr">
         <is>
@@ -4010,14 +4037,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I52" s="11" t="inlineStr"/>
+      <c r="I52" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J52" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
         </is>
       </c>
       <c r="K52" s="11" t="inlineStr"/>
-      <c r="L52" s="11" t="inlineStr"/>
+      <c r="L52" s="11" t="inlineStr">
+        <is>
+          <t>66126805997</t>
+        </is>
+      </c>
       <c r="M52" s="11" t="inlineStr"/>
       <c r="N52" s="11" t="inlineStr">
         <is>
@@ -4072,14 +4107,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I53" s="11" t="inlineStr"/>
+      <c r="I53" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J53" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
         </is>
       </c>
       <c r="K53" s="11" t="inlineStr"/>
-      <c r="L53" s="11" t="inlineStr"/>
+      <c r="L53" s="11" t="inlineStr">
+        <is>
+          <t>66126805997</t>
+        </is>
+      </c>
       <c r="M53" s="11" t="inlineStr"/>
       <c r="N53" s="11" t="inlineStr">
         <is>
@@ -5896,7 +5939,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I81" s="11" t="inlineStr"/>
+      <c r="I81" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J81" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -5905,7 +5952,7 @@
       <c r="K81" s="11" t="inlineStr"/>
       <c r="L81" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5767</t>
+          <t>FCC YGOHUF5767, 66129312543[M 스포츠], 66129312524[기본형], 66129312539[럭셔리 라인], 66129312532[스포츠 라인]</t>
         </is>
       </c>
       <c r="M81" s="11" t="inlineStr"/>
@@ -6226,7 +6273,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I86" s="11" t="inlineStr"/>
+      <c r="I86" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J86" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -6235,7 +6286,7 @@
       <c r="K86" s="11" t="inlineStr"/>
       <c r="L86" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A[4버튼]</t>
+          <t>FCC N5F-ID21A[4버튼], 66128708356[M 스포츠], 66128708340[기본형], 66128708372[인디비주얼]</t>
         </is>
       </c>
       <c r="M86" s="11" t="inlineStr"/>
@@ -6292,7 +6343,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I87" s="11" t="inlineStr"/>
+      <c r="I87" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J87" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -6301,7 +6356,7 @@
       <c r="K87" s="11" t="inlineStr"/>
       <c r="L87" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128708356[M 스포츠], 66128708340[기본형], 66128708372[인디비주얼]</t>
         </is>
       </c>
       <c r="M87" s="11" t="inlineStr"/>
@@ -6820,7 +6875,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I95" s="11" t="inlineStr"/>
+      <c r="I95" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J95" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -6886,7 +6945,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I96" s="11" t="inlineStr"/>
+      <c r="I96" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J96" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -7604,7 +7667,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I107" s="11" t="inlineStr"/>
+      <c r="I107" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J107" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -7613,7 +7680,7 @@
       <c r="K107" s="11" t="inlineStr"/>
       <c r="L107" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5662[4버튼]</t>
+          <t>FCC YGOHUF5662[4버튼], 66128723582[M 스포츠], 66129254893[기본형], 66129254909[럭셔리 라인], 66129254897[모던 라인], 66129254901[스포츠 라인]</t>
         </is>
       </c>
       <c r="M107" s="11" t="inlineStr"/>
@@ -8656,7 +8723,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I123" s="11" t="inlineStr"/>
+      <c r="I123" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J123" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -8722,7 +8793,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I124" s="11" t="inlineStr"/>
+      <c r="I124" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J124" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -8788,7 +8863,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I125" s="11" t="inlineStr"/>
+      <c r="I125" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J125" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -9653,7 +9732,11 @@
         </is>
       </c>
       <c r="K138" s="11" t="inlineStr"/>
-      <c r="L138" s="11" t="inlineStr"/>
+      <c r="L138" s="11" t="inlineStr">
+        <is>
+          <t>66126933076</t>
+        </is>
+      </c>
       <c r="M138" s="11" t="inlineStr"/>
       <c r="N138" s="11" t="inlineStr">
         <is>
@@ -9717,7 +9800,7 @@
       <c r="K139" s="11" t="inlineStr"/>
       <c r="L139" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK47[4버튼]</t>
+          <t>FCC KR55WK47[4버튼], 66126933076</t>
         </is>
       </c>
       <c r="M139" s="11" t="inlineStr"/>
@@ -9774,7 +9857,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I140" s="11" t="inlineStr"/>
+      <c r="I140" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J140" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -9783,7 +9870,7 @@
       <c r="K140" s="11" t="inlineStr"/>
       <c r="L140" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK47993</t>
+          <t>FCC KR55WK47993, 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M140" s="11" t="inlineStr"/>
@@ -9840,7 +9927,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I141" s="11" t="inlineStr"/>
+      <c r="I141" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J141" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -9849,7 +9940,7 @@
       <c r="K141" s="11" t="inlineStr"/>
       <c r="L141" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK47</t>
+          <t>FCC KR55WK47, 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M141" s="11" t="inlineStr"/>
@@ -9906,7 +9997,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I142" s="11" t="n"/>
+      <c r="I142" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J142" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -9915,7 +10010,7 @@
       <c r="K142" s="11" t="n"/>
       <c r="L142" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49123, FCC KR55WK49127[리모컨키]</t>
+          <t>FCC KR55WK49123, FCC KR55WK49127[리모컨키], 66126986584, 66129268487[컴포트액세스]</t>
         </is>
       </c>
       <c r="M142" s="11" t="n"/>
@@ -9972,7 +10067,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I143" s="11" t="n"/>
+      <c r="I143" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J143" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -9981,7 +10080,7 @@
       <c r="K143" s="11" t="n"/>
       <c r="L143" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49123, FCC KR55WK49127[리모컨키]</t>
+          <t>FCC KR55WK49123, FCC KR55WK49127[리모컨키], 66126986584, 66129268487[컴포트액세스]</t>
         </is>
       </c>
       <c r="M143" s="11" t="n"/>
@@ -10170,7 +10269,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I146" s="11" t="inlineStr"/>
+      <c r="I146" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J146" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -10179,7 +10282,7 @@
       <c r="K146" s="11" t="inlineStr"/>
       <c r="L146" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127[리모컨키], FCC KR55WK49147[컴포트액세스]</t>
+          <t>FCC KR55WK49127[리모컨키], FCC KR55WK49147[컴포트액세스], 66126986584, 66129268487[컴포트액세스]</t>
         </is>
       </c>
       <c r="M146" s="11" t="inlineStr"/>
@@ -10236,7 +10339,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I147" s="11" t="n"/>
+      <c r="I147" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J147" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -10245,7 +10352,7 @@
       <c r="K147" s="11" t="inlineStr"/>
       <c r="L147" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127[리모컨키]</t>
+          <t>FCC KR55WK49127[리모컨키], 66126986584, 66129268487[컴포트액세스]</t>
         </is>
       </c>
       <c r="M147" s="11" t="inlineStr"/>
@@ -10368,7 +10475,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I149" s="11" t="inlineStr"/>
+      <c r="I149" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J149" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -10377,7 +10488,7 @@
       <c r="K149" s="11" t="inlineStr"/>
       <c r="L149" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49863</t>
+          <t>FCC KR55WK49863, 66129284934[럭셔리 라인], 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M149" s="11" t="inlineStr"/>
@@ -10434,7 +10545,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I150" s="11" t="n"/>
+      <c r="I150" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J150" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -10443,7 +10558,7 @@
       <c r="K150" s="11" t="n"/>
       <c r="L150" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49863</t>
+          <t>FCC KR55WK49863, 66129284934[럭셔리 라인], 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M150" s="11" t="n"/>
@@ -10500,7 +10615,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I151" s="11" t="n"/>
+      <c r="I151" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J151" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -10509,7 +10628,7 @@
       <c r="K151" s="11" t="n"/>
       <c r="L151" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49863</t>
+          <t>FCC KR55WK49863, 66129284934[럭셔리 라인], 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M151" s="11" t="n"/>
@@ -10566,7 +10685,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I152" s="11" t="inlineStr"/>
+      <c r="I152" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J152" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -10575,7 +10698,7 @@
       <c r="K152" s="11" t="inlineStr"/>
       <c r="L152" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49863</t>
+          <t>FCC KR55WK49863, 66129284934[럭셔리 라인], 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M152" s="11" t="inlineStr"/>
@@ -10632,7 +10755,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I153" s="11" t="inlineStr"/>
+      <c r="I153" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J153" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -10641,7 +10768,7 @@
       <c r="K153" s="11" t="inlineStr"/>
       <c r="L153" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5767[4버튼]</t>
+          <t>FCC YGOHUF5767[4버튼], 66129284934[럭셔리 라인], 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M153" s="11" t="inlineStr"/>
@@ -10698,7 +10825,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I154" s="11" t="inlineStr"/>
+      <c r="I154" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J154" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -10707,7 +10838,7 @@
       <c r="K154" s="11" t="inlineStr"/>
       <c r="L154" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5767</t>
+          <t>FCC YGOHUF5767, 66129284934[럭셔리 라인], 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M154" s="11" t="inlineStr"/>
@@ -10764,7 +10895,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I155" s="11" t="inlineStr"/>
+      <c r="I155" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J155" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -10773,7 +10908,7 @@
       <c r="K155" s="11" t="inlineStr"/>
       <c r="L155" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5767</t>
+          <t>FCC YGOHUF5767, 66129284934[럭셔리 라인], 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M155" s="11" t="inlineStr"/>
@@ -10830,7 +10965,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I156" s="11" t="inlineStr"/>
+      <c r="I156" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J156" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -10839,7 +10978,7 @@
       <c r="K156" s="11" t="inlineStr"/>
       <c r="L156" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49863, FCC YGOHUF5767</t>
+          <t>FCC KR55WK49863, FCC YGOHUF5767, 66129284934[럭셔리 라인], 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M156" s="11" t="inlineStr"/>
@@ -11028,14 +11167,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I159" s="11" t="n"/>
+      <c r="I159" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J159" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
         </is>
       </c>
       <c r="K159" s="11" t="n"/>
-      <c r="L159" s="11" t="n"/>
+      <c r="L159" s="11" t="inlineStr">
+        <is>
+          <t>66129284934[럭셔리 라인], 66129259720[컴포트액세스]</t>
+        </is>
+      </c>
       <c r="M159" s="11" t="n"/>
       <c r="N159" s="11" t="inlineStr">
         <is>
@@ -11090,14 +11237,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I160" s="11" t="n"/>
+      <c r="I160" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J160" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
         </is>
       </c>
       <c r="K160" s="11" t="n"/>
-      <c r="L160" s="11" t="n"/>
+      <c r="L160" s="11" t="inlineStr">
+        <is>
+          <t>66129284934[럭셔리 라인], 66129259720[컴포트액세스]</t>
+        </is>
+      </c>
       <c r="M160" s="11" t="n"/>
       <c r="N160" s="11" t="inlineStr">
         <is>
@@ -11284,7 +11439,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I163" s="11" t="inlineStr"/>
+      <c r="I163" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J163" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -11293,7 +11452,7 @@
       <c r="K163" s="11" t="inlineStr"/>
       <c r="L163" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5662, FCC KR55WK49863</t>
+          <t>FCC YGOHUF5662, FCC KR55WK49863, 66129284934[럭셔리 라인], 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M163" s="11" t="inlineStr"/>
@@ -11416,7 +11575,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I165" s="11" t="inlineStr"/>
+      <c r="I165" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J165" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -11425,7 +11588,7 @@
       <c r="K165" s="11" t="inlineStr"/>
       <c r="L165" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5662</t>
+          <t>FCC YGOHUF5662, 66129284934[럭셔리 라인], 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M165" s="11" t="inlineStr"/>
@@ -11680,7 +11843,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I169" s="11" t="n"/>
+      <c r="I169" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J169" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -11689,7 +11856,7 @@
       <c r="K169" s="11" t="n"/>
       <c r="L169" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128717527[M 스포츠], 66128717511[기본형], 66128779008[디스플레이키], 66128717535[인디비주얼]</t>
         </is>
       </c>
       <c r="M169" s="11" t="n"/>
@@ -11746,7 +11913,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I170" s="11" t="n"/>
+      <c r="I170" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J170" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -11755,7 +11926,7 @@
       <c r="K170" s="11" t="n"/>
       <c r="L170" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128717527[M 스포츠], 66128717511[기본형], 66128779008[디스플레이키], 66128717535[인디비주얼]</t>
         </is>
       </c>
       <c r="M170" s="11" t="n"/>
@@ -12830,7 +13001,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I186" s="11" t="inlineStr"/>
+      <c r="I186" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J186" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -12839,7 +13014,7 @@
       <c r="K186" s="11" t="inlineStr"/>
       <c r="L186" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK47993[3버튼]</t>
+          <t>FCC KR55WK47993[3버튼], 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M186" s="11" t="inlineStr"/>
@@ -12896,7 +13071,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I187" s="11" t="inlineStr"/>
+      <c r="I187" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J187" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -12905,7 +13084,7 @@
       <c r="K187" s="11" t="inlineStr"/>
       <c r="L187" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK47[4버튼]</t>
+          <t>FCC KR55WK47[4버튼], 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M187" s="11" t="inlineStr"/>
@@ -12962,7 +13141,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I188" s="11" t="n"/>
+      <c r="I188" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J188" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -12971,7 +13154,7 @@
       <c r="K188" s="11" t="n"/>
       <c r="L188" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127[리모컨키], FCC KR55WK49147[컴포트액세스]</t>
+          <t>FCC KR55WK49127[리모컨키], FCC KR55WK49147[컴포트액세스], 66126986584, 66129268487[컴포트액세스]</t>
         </is>
       </c>
       <c r="M188" s="11" t="n"/>
@@ -13028,7 +13211,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I189" s="11" t="n"/>
+      <c r="I189" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J189" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -13037,7 +13224,7 @@
       <c r="K189" s="11" t="n"/>
       <c r="L189" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127[리모컨키], FCC KR55WK49147[컴포트액세스]</t>
+          <t>FCC KR55WK49127[리모컨키], FCC KR55WK49147[컴포트액세스], 66126986584, 66129268487[컴포트액세스]</t>
         </is>
       </c>
       <c r="M189" s="11" t="n"/>
@@ -13094,7 +13281,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I190" s="11" t="n"/>
+      <c r="I190" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J190" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -13103,7 +13294,7 @@
       <c r="K190" s="11" t="n"/>
       <c r="L190" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49147[컴포트액세스]</t>
+          <t>FCC KR55WK49147[컴포트액세스], 66126986584, 66129268487[컴포트액세스]</t>
         </is>
       </c>
       <c r="M190" s="11" t="n"/>
@@ -13160,7 +13351,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I191" s="11" t="n"/>
+      <c r="I191" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J191" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -13169,7 +13364,7 @@
       <c r="K191" s="11" t="n"/>
       <c r="L191" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49147[컴포트액세스]</t>
+          <t>FCC KR55WK49147[컴포트액세스], 66126986584, 66129268487[컴포트액세스]</t>
         </is>
       </c>
       <c r="M191" s="11" t="n"/>
@@ -13226,7 +13421,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I192" s="11" t="inlineStr"/>
+      <c r="I192" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J192" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -13235,7 +13434,7 @@
       <c r="K192" s="11" t="inlineStr"/>
       <c r="L192" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127[리모컨키]</t>
+          <t>FCC KR55WK49127[리모컨키], 66126986584, 66129268487[컴포트액세스]</t>
         </is>
       </c>
       <c r="M192" s="11" t="inlineStr"/>
@@ -13292,7 +13491,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I193" s="11" t="inlineStr"/>
+      <c r="I193" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J193" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -13301,7 +13504,7 @@
       <c r="K193" s="11" t="inlineStr"/>
       <c r="L193" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127[리모컨키]</t>
+          <t>FCC KR55WK49127[리모컨키], 66126986584, 66129268487[컴포트액세스]</t>
         </is>
       </c>
       <c r="M193" s="11" t="inlineStr"/>
@@ -13424,7 +13627,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I195" s="11" t="n"/>
+      <c r="I195" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J195" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -13433,7 +13640,7 @@
       <c r="K195" s="11" t="n"/>
       <c r="L195" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49863, FCC YGOHUF5662</t>
+          <t>FCC KR55WK49863, FCC YGOHUF5662, 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M195" s="11" t="n"/>
@@ -13490,7 +13697,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I196" s="11" t="n"/>
+      <c r="I196" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J196" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -13499,7 +13710,7 @@
       <c r="K196" s="11" t="n"/>
       <c r="L196" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49863, FCC YGOHUF5662</t>
+          <t>FCC KR55WK49863, FCC YGOHUF5662, 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M196" s="11" t="n"/>
@@ -13556,7 +13767,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I197" s="11" t="inlineStr"/>
+      <c r="I197" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J197" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -13565,7 +13780,7 @@
       <c r="K197" s="11" t="inlineStr"/>
       <c r="L197" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5767</t>
+          <t>FCC YGOHUF5767, 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M197" s="11" t="inlineStr"/>
@@ -13622,7 +13837,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I198" s="11" t="inlineStr"/>
+      <c r="I198" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J198" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -13631,7 +13850,7 @@
       <c r="K198" s="11" t="inlineStr"/>
       <c r="L198" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5767</t>
+          <t>FCC YGOHUF5767, 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M198" s="11" t="inlineStr"/>
@@ -13688,7 +13907,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I199" s="11" t="inlineStr"/>
+      <c r="I199" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J199" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -13697,7 +13920,7 @@
       <c r="K199" s="11" t="inlineStr"/>
       <c r="L199" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5767</t>
+          <t>FCC YGOHUF5767, 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M199" s="11" t="inlineStr"/>
@@ -13754,7 +13977,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I200" s="11" t="inlineStr"/>
+      <c r="I200" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J200" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -13763,7 +13990,7 @@
       <c r="K200" s="11" t="inlineStr"/>
       <c r="L200" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5767</t>
+          <t>FCC YGOHUF5767, 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M200" s="11" t="inlineStr"/>
@@ -13820,7 +14047,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I201" s="11" t="inlineStr"/>
+      <c r="I201" s="11" t="inlineStr">
+        <is>
+          <t>51217293906[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J201" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -13829,7 +14060,7 @@
       <c r="K201" s="11" t="inlineStr"/>
       <c r="L201" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5662, FCC YGOHUF5767</t>
+          <t>FCC YGOHUF5662, FCC YGOHUF5767, 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M201" s="11" t="inlineStr"/>
@@ -14018,7 +14249,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I204" s="11" t="n"/>
+      <c r="I204" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J204" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -14027,7 +14262,7 @@
       <c r="K204" s="11" t="n"/>
       <c r="L204" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128717527[M 스포츠], 66128779004[디스플레이키]</t>
         </is>
       </c>
       <c r="M204" s="11" t="n"/>
@@ -14084,7 +14319,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I205" s="11" t="n"/>
+      <c r="I205" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J205" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -14093,7 +14332,7 @@
       <c r="K205" s="11" t="n"/>
       <c r="L205" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128717527[M 스포츠], 66128779004[디스플레이키]</t>
         </is>
       </c>
       <c r="M205" s="11" t="n"/>
@@ -14623,7 +14862,11 @@
         </is>
       </c>
       <c r="K213" s="11" t="inlineStr"/>
-      <c r="L213" s="11" t="inlineStr"/>
+      <c r="L213" s="11" t="inlineStr">
+        <is>
+          <t>66126933076</t>
+        </is>
+      </c>
       <c r="M213" s="11" t="inlineStr"/>
       <c r="N213" s="11" t="inlineStr">
         <is>
@@ -14687,7 +14930,7 @@
       <c r="K214" s="11" t="inlineStr"/>
       <c r="L214" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK47[4버튼]</t>
+          <t>FCC KR55WK47[4버튼], 66126933076</t>
         </is>
       </c>
       <c r="M214" s="11" t="inlineStr"/>
@@ -14744,7 +14987,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I215" s="11" t="inlineStr"/>
+      <c r="I215" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J215" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -14753,7 +15000,7 @@
       <c r="K215" s="11" t="inlineStr"/>
       <c r="L215" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK47993</t>
+          <t>FCC KR55WK47993, 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M215" s="11" t="inlineStr"/>
@@ -14810,7 +15057,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I216" s="11" t="inlineStr"/>
+      <c r="I216" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J216" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -14819,7 +15070,7 @@
       <c r="K216" s="11" t="inlineStr"/>
       <c r="L216" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK47, FCC LX8FZV</t>
+          <t>FCC KR55WK47, FCC LX8FZV, 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M216" s="11" t="inlineStr"/>
@@ -14876,7 +15127,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I217" s="11" t="n"/>
+      <c r="I217" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J217" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -14885,7 +15140,7 @@
       <c r="K217" s="11" t="n"/>
       <c r="L217" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127[리모컨키], FCC KR55WK49147[컴포트액세스]</t>
+          <t>FCC KR55WK49127[리모컨키], FCC KR55WK49147[컴포트액세스], 66126986584, 66129268487[컴포트액세스]</t>
         </is>
       </c>
       <c r="M217" s="11" t="n"/>
@@ -14942,7 +15197,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I218" s="11" t="n"/>
+      <c r="I218" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J218" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -14951,7 +15210,7 @@
       <c r="K218" s="11" t="n"/>
       <c r="L218" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127[리모컨키], FCC KR55WK49147[컴포트액세스]</t>
+          <t>FCC KR55WK49127[리모컨키], FCC KR55WK49147[컴포트액세스], 66126986584, 66129268487[컴포트액세스]</t>
         </is>
       </c>
       <c r="M218" s="11" t="n"/>
@@ -15140,7 +15399,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I221" s="11" t="inlineStr"/>
+      <c r="I221" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J221" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -15149,7 +15412,7 @@
       <c r="K221" s="11" t="inlineStr"/>
       <c r="L221" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127[리모컨키]</t>
+          <t>FCC KR55WK49127[리모컨키], 66126986584, 66129268487[컴포트액세스]</t>
         </is>
       </c>
       <c r="M221" s="11" t="inlineStr"/>
@@ -15206,7 +15469,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I222" s="11" t="inlineStr"/>
+      <c r="I222" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J222" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -15215,7 +15482,7 @@
       <c r="K222" s="11" t="inlineStr"/>
       <c r="L222" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127[리모컨키]</t>
+          <t>FCC KR55WK49127[리모컨키], 66126986584, 66129268487[컴포트액세스]</t>
         </is>
       </c>
       <c r="M222" s="11" t="inlineStr"/>
@@ -15272,7 +15539,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I223" s="11" t="inlineStr"/>
+      <c r="I223" s="11" t="inlineStr">
+        <is>
+          <t>51217227123[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J223" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -15281,7 +15552,7 @@
       <c r="K223" s="11" t="inlineStr"/>
       <c r="L223" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49863, FCC YGOHUF5662</t>
+          <t>FCC KR55WK49863, FCC YGOHUF5662, 66129259716[컴포트액세스]</t>
         </is>
       </c>
       <c r="M223" s="11" t="inlineStr"/>
@@ -15338,7 +15609,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I224" s="11" t="n"/>
+      <c r="I224" s="11" t="inlineStr">
+        <is>
+          <t>51217227123[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J224" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -15347,7 +15622,7 @@
       <c r="K224" s="11" t="n"/>
       <c r="L224" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5662</t>
+          <t>FCC YGOHUF5662, 66129259716[컴포트액세스]</t>
         </is>
       </c>
       <c r="M224" s="11" t="n"/>
@@ -15404,7 +15679,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I225" s="11" t="n"/>
+      <c r="I225" s="11" t="inlineStr">
+        <is>
+          <t>51217227123[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J225" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -15413,7 +15692,7 @@
       <c r="K225" s="11" t="n"/>
       <c r="L225" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5662</t>
+          <t>FCC YGOHUF5662, 66129259716[컴포트액세스]</t>
         </is>
       </c>
       <c r="M225" s="11" t="n"/>
@@ -15998,7 +16277,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I234" s="11" t="inlineStr"/>
+      <c r="I234" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J234" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -16007,7 +16290,7 @@
       <c r="K234" s="11" t="inlineStr"/>
       <c r="L234" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128717527[M 스포츠], 66128717511[기본형], 66128779008[디스플레이키]</t>
         </is>
       </c>
       <c r="M234" s="11" t="inlineStr"/>
@@ -16064,7 +16347,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I235" s="11" t="n"/>
+      <c r="I235" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J235" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -16073,7 +16360,7 @@
       <c r="K235" s="11" t="n"/>
       <c r="L235" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128717527[M 스포츠], 66128717511[기본형], 66128779008[디스플레이키]</t>
         </is>
       </c>
       <c r="M235" s="11" t="n"/>
@@ -16130,7 +16417,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I236" s="11" t="n"/>
+      <c r="I236" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J236" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -16139,7 +16430,7 @@
       <c r="K236" s="11" t="n"/>
       <c r="L236" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128717527[M 스포츠], 66128717511[기본형], 66128779008[디스플레이키]</t>
         </is>
       </c>
       <c r="M236" s="11" t="n"/>
@@ -16390,7 +16681,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I240" s="11" t="inlineStr"/>
+      <c r="I240" s="11" t="inlineStr">
+        <is>
+          <t>51217227123[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J240" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -16399,7 +16694,7 @@
       <c r="K240" s="11" t="inlineStr"/>
       <c r="L240" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49863</t>
+          <t>FCC KR55WK49863, 66129259716[컴포트액세스]</t>
         </is>
       </c>
       <c r="M240" s="11" t="inlineStr"/>
@@ -16456,7 +16751,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I241" s="11" t="n"/>
+      <c r="I241" s="11" t="inlineStr">
+        <is>
+          <t>51217227123[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J241" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -16465,7 +16764,7 @@
       <c r="K241" s="11" t="n"/>
       <c r="L241" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49863, FCC YGOHUF5662</t>
+          <t>FCC KR55WK49863, FCC YGOHUF5662, 66129259716[컴포트액세스]</t>
         </is>
       </c>
       <c r="M241" s="11" t="n"/>
@@ -16522,7 +16821,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I242" s="11" t="n"/>
+      <c r="I242" s="11" t="inlineStr">
+        <is>
+          <t>51217227123[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J242" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -16531,7 +16834,7 @@
       <c r="K242" s="11" t="n"/>
       <c r="L242" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49863, FCC YGOHUF5662</t>
+          <t>FCC KR55WK49863, FCC YGOHUF5662, 66129259716[컴포트액세스]</t>
         </is>
       </c>
       <c r="M242" s="11" t="n"/>
@@ -16588,7 +16891,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I243" s="11" t="inlineStr"/>
+      <c r="I243" s="11" t="inlineStr">
+        <is>
+          <t>51217227123[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J243" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -16597,7 +16904,7 @@
       <c r="K243" s="11" t="inlineStr"/>
       <c r="L243" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5767</t>
+          <t>FCC YGOHUF5767, 66129259716[컴포트액세스]</t>
         </is>
       </c>
       <c r="M243" s="11" t="inlineStr"/>
@@ -16654,7 +16961,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I244" s="11" t="inlineStr"/>
+      <c r="I244" s="11" t="inlineStr">
+        <is>
+          <t>51217227123[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J244" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -16663,7 +16974,7 @@
       <c r="K244" s="11" t="inlineStr"/>
       <c r="L244" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5662</t>
+          <t>FCC YGOHUF5662, 66129259716[컴포트액세스]</t>
         </is>
       </c>
       <c r="M244" s="11" t="inlineStr"/>
@@ -17190,7 +17501,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I252" s="11" t="inlineStr"/>
+      <c r="I252" s="11" t="inlineStr">
+        <is>
+          <t>51217066345[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J252" s="11" t="inlineStr">
         <is>
           <t>HU92[비상키]</t>
@@ -17199,7 +17514,7 @@
       <c r="K252" s="11" t="inlineStr"/>
       <c r="L252" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8766S</t>
+          <t>FCC LX8766S, 66126959045, 66126959060[컴포트액세스]</t>
         </is>
       </c>
       <c r="M252" s="11" t="inlineStr"/>
@@ -17256,7 +17571,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I253" s="11" t="inlineStr"/>
+      <c r="I253" s="11" t="inlineStr">
+        <is>
+          <t>51217066345[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J253" s="11" t="inlineStr">
         <is>
           <t>HU92[비상키]</t>
@@ -17265,7 +17584,7 @@
       <c r="K253" s="11" t="inlineStr"/>
       <c r="L253" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8766S</t>
+          <t>FCC LX8766S, 66126959045, 66126959060[컴포트액세스]</t>
         </is>
       </c>
       <c r="M253" s="11" t="inlineStr"/>
@@ -17322,7 +17641,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I254" s="11" t="n"/>
+      <c r="I254" s="11" t="inlineStr">
+        <is>
+          <t>51217066345[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J254" s="11" t="inlineStr">
         <is>
           <t>HU92[비상키]</t>
@@ -17331,7 +17654,7 @@
       <c r="K254" s="11" t="n"/>
       <c r="L254" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8766S</t>
+          <t>FCC LX8766S, 66126959045, 66126959060[컴포트액세스]</t>
         </is>
       </c>
       <c r="M254" s="11" t="n"/>
@@ -17388,7 +17711,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I255" s="11" t="n"/>
+      <c r="I255" s="11" t="inlineStr">
+        <is>
+          <t>51217066345[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J255" s="11" t="inlineStr">
         <is>
           <t>HU92[비상키]</t>
@@ -17397,7 +17724,7 @@
       <c r="K255" s="11" t="n"/>
       <c r="L255" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8766S</t>
+          <t>FCC LX8766S, 66126959045, 66126959060[컴포트액세스]</t>
         </is>
       </c>
       <c r="M255" s="11" t="n"/>
@@ -17454,7 +17781,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I256" s="11" t="inlineStr"/>
+      <c r="I256" s="11" t="inlineStr">
+        <is>
+          <t>51217066345[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J256" s="11" t="inlineStr">
         <is>
           <t>HU92[비상키]</t>
@@ -17463,7 +17794,7 @@
       <c r="K256" s="11" t="inlineStr"/>
       <c r="L256" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8766S</t>
+          <t>FCC LX8766S, 66126959045, 66126959060[컴포트액세스]</t>
         </is>
       </c>
       <c r="M256" s="11" t="inlineStr"/>
@@ -17520,7 +17851,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I257" s="11" t="inlineStr"/>
+      <c r="I257" s="11" t="inlineStr">
+        <is>
+          <t>51217066345[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J257" s="11" t="inlineStr">
         <is>
           <t>HU92[비상키]</t>
@@ -17529,7 +17864,7 @@
       <c r="K257" s="11" t="inlineStr"/>
       <c r="L257" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8766S</t>
+          <t>FCC LX8766S, 66126959045, 66126959060[컴포트액세스]</t>
         </is>
       </c>
       <c r="M257" s="11" t="inlineStr"/>
@@ -17586,7 +17921,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I258" s="11" t="inlineStr"/>
+      <c r="I258" s="11" t="inlineStr">
+        <is>
+          <t>51217066345[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J258" s="11" t="inlineStr">
         <is>
           <t>HU92[비상키]</t>
@@ -17595,7 +17934,7 @@
       <c r="K258" s="11" t="inlineStr"/>
       <c r="L258" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8766S</t>
+          <t>FCC LX8766S, 66126959045, 66126959060[컴포트액세스]</t>
         </is>
       </c>
       <c r="M258" s="11" t="inlineStr"/>
@@ -17982,7 +18321,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I264" s="11" t="inlineStr"/>
+      <c r="I264" s="11" t="inlineStr">
+        <is>
+          <t>51217227123[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J264" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -17991,7 +18334,7 @@
       <c r="K264" s="11" t="inlineStr"/>
       <c r="L264" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5767</t>
+          <t>FCC YGOHUF5767, 66129259716[컴포트액세스]</t>
         </is>
       </c>
       <c r="M264" s="11" t="inlineStr"/>
@@ -18048,7 +18391,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I265" s="11" t="inlineStr"/>
+      <c r="I265" s="11" t="inlineStr">
+        <is>
+          <t>51217227123[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J265" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -18057,7 +18404,7 @@
       <c r="K265" s="11" t="inlineStr"/>
       <c r="L265" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5767</t>
+          <t>FCC YGOHUF5767, 66129259716[컴포트액세스]</t>
         </is>
       </c>
       <c r="M265" s="11" t="inlineStr"/>
@@ -18114,7 +18461,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I266" s="11" t="inlineStr"/>
+      <c r="I266" s="11" t="inlineStr">
+        <is>
+          <t>51217227123[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J266" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -18123,7 +18474,7 @@
       <c r="K266" s="11" t="inlineStr"/>
       <c r="L266" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5767</t>
+          <t>FCC YGOHUF5767, 66129259716[컴포트액세스]</t>
         </is>
       </c>
       <c r="M266" s="11" t="inlineStr"/>
@@ -18378,7 +18729,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I270" s="11" t="inlineStr"/>
+      <c r="I270" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J270" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -18387,7 +18742,7 @@
       <c r="K270" s="11" t="inlineStr"/>
       <c r="L270" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128808897[M 스포츠], 66128808880[기본형], 66128806245[디스플레이키], 66128808905[인디비주얼]</t>
         </is>
       </c>
       <c r="M270" s="11" t="inlineStr"/>
@@ -18444,7 +18799,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I271" s="11" t="n"/>
+      <c r="I271" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J271" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -18453,7 +18812,7 @@
       <c r="K271" s="11" t="n"/>
       <c r="L271" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128717527[M 스포츠], 66128717511[기본형], 66128779008[디스플레이키], 66128717535[인디비주얼]</t>
         </is>
       </c>
       <c r="M271" s="11" t="n"/>
@@ -18510,7 +18869,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I272" s="11" t="n"/>
+      <c r="I272" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J272" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -18519,7 +18882,7 @@
       <c r="K272" s="11" t="n"/>
       <c r="L272" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128717527[M 스포츠], 66128717511[기본형], 66128779008[디스플레이키], 66128717535[인디비주얼]</t>
         </is>
       </c>
       <c r="M272" s="11" t="n"/>
@@ -18576,7 +18939,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I273" s="11" t="inlineStr"/>
+      <c r="I273" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J273" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -18585,7 +18952,7 @@
       <c r="K273" s="11" t="inlineStr"/>
       <c r="L273" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128717527[M 스포츠], 66128717511[기본형], 66128779008[디스플레이키], 66128717535[인디비주얼]</t>
         </is>
       </c>
       <c r="M273" s="11" t="inlineStr"/>
@@ -19500,7 +19867,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I287" s="11" t="inlineStr"/>
+      <c r="I287" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J287" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -19509,7 +19880,7 @@
       <c r="K287" s="11" t="inlineStr"/>
       <c r="L287" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128708348, 66128708364[M 스포츠], 66129855654[디스플레이키], 66128708372[인디비주얼]</t>
         </is>
       </c>
       <c r="M287" s="11" t="inlineStr"/>
@@ -20754,7 +21125,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I306" s="11" t="inlineStr"/>
+      <c r="I306" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J306" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -20763,7 +21138,7 @@
       <c r="K306" s="11" t="inlineStr"/>
       <c r="L306" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127[리모컨키]</t>
+          <t>FCC KR55WK49127[리모컨키], 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M306" s="11" t="inlineStr"/>
@@ -20886,7 +21261,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I308" s="11" t="inlineStr"/>
+      <c r="I308" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J308" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -20895,7 +21274,7 @@
       <c r="K308" s="11" t="inlineStr"/>
       <c r="L308" s="11" t="inlineStr">
         <is>
-          <t>FCC NBGIDGNG1</t>
+          <t>FCC NBGIDGNG1, 66126805998[M 스포츠, 해외 공용 품번], 66126805990[기본형, 해외 공용 품번]</t>
         </is>
       </c>
       <c r="M308" s="11" t="inlineStr"/>
@@ -20952,7 +21331,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I309" s="11" t="inlineStr"/>
+      <c r="I309" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J309" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -20961,7 +21344,7 @@
       <c r="K309" s="11" t="inlineStr"/>
       <c r="L309" s="11" t="inlineStr">
         <is>
-          <t>FCC NBGIDGNG1</t>
+          <t>FCC NBGIDGNG1, 66126805998[M 스포츠, 해외 공용 품번], 66126805990[기본형, 해외 공용 품번]</t>
         </is>
       </c>
       <c r="M309" s="11" t="inlineStr"/>
@@ -21018,7 +21401,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I310" s="11" t="inlineStr"/>
+      <c r="I310" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J310" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -21027,7 +21414,7 @@
       <c r="K310" s="11" t="inlineStr"/>
       <c r="L310" s="11" t="inlineStr">
         <is>
-          <t>FCC NBGIDGNG1</t>
+          <t>FCC NBGIDGNG1, 66126805998[M 스포츠, 해외 공용 품번], 66126805990[기본형, 해외 공용 품번]</t>
         </is>
       </c>
       <c r="M310" s="11" t="inlineStr"/>
@@ -21084,14 +21471,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I311" s="11" t="inlineStr"/>
+      <c r="I311" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J311" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
         </is>
       </c>
       <c r="K311" s="11" t="inlineStr"/>
-      <c r="L311" s="11" t="n"/>
+      <c r="L311" s="11" t="inlineStr">
+        <is>
+          <t>66126805998[M 스포츠, 해외 공용 품번], 66126805990[기본형, 해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="M311" s="11" t="inlineStr"/>
       <c r="N311" s="11" t="inlineStr">
         <is>
@@ -21146,14 +21541,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I312" s="11" t="inlineStr"/>
+      <c r="I312" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J312" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
         </is>
       </c>
       <c r="K312" s="11" t="inlineStr"/>
-      <c r="L312" s="11" t="n"/>
+      <c r="L312" s="11" t="inlineStr">
+        <is>
+          <t>66126805990[기본형, 해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="M312" s="11" t="inlineStr"/>
       <c r="N312" s="11" t="inlineStr">
         <is>
@@ -21876,7 +22279,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I323" s="11" t="inlineStr"/>
+      <c r="I323" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J323" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -21885,7 +22292,7 @@
       <c r="K323" s="11" t="inlineStr"/>
       <c r="L323" s="11" t="inlineStr">
         <is>
-          <t>FCC NBGIDGNG1</t>
+          <t>FCC NBGIDGNG1, 66126805998[M 스포츠, 해외 공용 품번], 66126805990[기본형, 해외 공용 품번]</t>
         </is>
       </c>
       <c r="M323" s="11" t="inlineStr"/>
@@ -21942,7 +22349,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I324" s="11" t="inlineStr"/>
+      <c r="I324" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J324" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -21951,7 +22362,7 @@
       <c r="K324" s="11" t="inlineStr"/>
       <c r="L324" s="11" t="inlineStr">
         <is>
-          <t>FCC NBGIDGNG1</t>
+          <t>FCC NBGIDGNG1, 66126805998[M 스포츠, 해외 공용 품번], 66126805990[기본형, 해외 공용 품번]</t>
         </is>
       </c>
       <c r="M324" s="11" t="inlineStr"/>
@@ -23014,7 +23425,11 @@
           <t>막대키</t>
         </is>
       </c>
-      <c r="I340" s="11" t="inlineStr"/>
+      <c r="I340" s="11" t="inlineStr">
+        <is>
+          <t>51217127047[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J340" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -23023,7 +23438,7 @@
       <c r="K340" s="11" t="inlineStr"/>
       <c r="L340" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8FZV</t>
+          <t>FCC LX8FZV, 66126955747[해외 공용 품번], 51218374933[적외선 리모컨]</t>
         </is>
       </c>
       <c r="M340" s="11" t="inlineStr"/>
@@ -23080,7 +23495,11 @@
           <t>막대키</t>
         </is>
       </c>
-      <c r="I341" s="11" t="inlineStr"/>
+      <c r="I341" s="11" t="inlineStr">
+        <is>
+          <t>51217127047[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J341" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -23089,7 +23508,7 @@
       <c r="K341" s="11" t="inlineStr"/>
       <c r="L341" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8FZV</t>
+          <t>FCC LX8FZV, 66126955747[해외 공용 품번], 51218374933[적외선 리모컨]</t>
         </is>
       </c>
       <c r="M341" s="11" t="inlineStr"/>
@@ -23146,14 +23565,22 @@
           <t>막대키</t>
         </is>
       </c>
-      <c r="I342" s="11" t="inlineStr"/>
+      <c r="I342" s="11" t="inlineStr">
+        <is>
+          <t>51217127047[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J342" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
         </is>
       </c>
       <c r="K342" s="11" t="inlineStr"/>
-      <c r="L342" s="11" t="inlineStr"/>
+      <c r="L342" s="11" t="inlineStr">
+        <is>
+          <t>66126955747[해외 공용 품번], 51218374933[적외선 리모컨]</t>
+        </is>
+      </c>
       <c r="M342" s="11" t="inlineStr"/>
       <c r="N342" s="11" t="inlineStr">
         <is>
@@ -23208,7 +23635,11 @@
           <t>막대키</t>
         </is>
       </c>
-      <c r="I343" s="11" t="inlineStr"/>
+      <c r="I343" s="11" t="inlineStr">
+        <is>
+          <t>51217127047[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J343" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -23217,7 +23648,7 @@
       <c r="K343" s="11" t="inlineStr"/>
       <c r="L343" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8FZV</t>
+          <t>FCC LX8FZV, 66126955747[해외 공용 품번], 51218374933[적외선 리모컨]</t>
         </is>
       </c>
       <c r="M343" s="11" t="inlineStr"/>
@@ -23274,14 +23705,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I344" s="11" t="inlineStr"/>
+      <c r="I344" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J344" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
         </is>
       </c>
       <c r="K344" s="11" t="inlineStr"/>
-      <c r="L344" s="11" t="inlineStr"/>
+      <c r="L344" s="11" t="inlineStr">
+        <is>
+          <t>66129259720[컴포트액세스]</t>
+        </is>
+      </c>
       <c r="M344" s="11" t="inlineStr"/>
       <c r="N344" s="11" t="inlineStr">
         <is>
@@ -23336,7 +23775,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I345" s="11" t="n"/>
+      <c r="I345" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J345" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -23345,7 +23788,7 @@
       <c r="K345" s="11" t="n"/>
       <c r="L345" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5662</t>
+          <t>FCC YGOHUF5662, 66129254893[기본형], 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M345" s="11" t="n"/>
@@ -23402,7 +23845,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I346" s="11" t="n"/>
+      <c r="I346" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J346" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -23411,7 +23858,7 @@
       <c r="K346" s="11" t="n"/>
       <c r="L346" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5662</t>
+          <t>FCC YGOHUF5662, 66129254893[기본형], 66129259720[컴포트액세스]</t>
         </is>
       </c>
       <c r="M346" s="11" t="n"/>
@@ -23600,7 +24047,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I349" s="11" t="n"/>
+      <c r="I349" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J349" s="11" t="inlineStr">
         <is>
           <t>HU100R</t>
@@ -23609,7 +24060,7 @@
       <c r="K349" s="11" t="inlineStr"/>
       <c r="L349" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5662, FCC KR55WK49863</t>
+          <t>FCC YGOHUF5662, FCC KR55WK49863, 66129254893[기본형]</t>
         </is>
       </c>
       <c r="M349" s="11" t="inlineStr"/>
@@ -23666,14 +24117,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I350" s="11" t="inlineStr"/>
+      <c r="I350" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J350" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
         </is>
       </c>
       <c r="K350" s="11" t="inlineStr"/>
-      <c r="L350" s="11" t="inlineStr"/>
+      <c r="L350" s="11" t="inlineStr">
+        <is>
+          <t>66129254893[기본형]</t>
+        </is>
+      </c>
       <c r="M350" s="11" t="inlineStr"/>
       <c r="N350" s="11" t="inlineStr">
         <is>
@@ -23728,14 +24187,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I351" s="11" t="inlineStr"/>
+      <c r="I351" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J351" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
         </is>
       </c>
       <c r="K351" s="11" t="inlineStr"/>
-      <c r="L351" s="11" t="n"/>
+      <c r="L351" s="11" t="inlineStr">
+        <is>
+          <t>66129254893[기본형]</t>
+        </is>
+      </c>
       <c r="M351" s="11" t="inlineStr"/>
       <c r="N351" s="11" t="inlineStr">
         <is>
@@ -23922,7 +24389,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I354" s="11" t="inlineStr"/>
+      <c r="I354" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J354" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -23931,7 +24402,7 @@
       <c r="K354" s="11" t="inlineStr"/>
       <c r="L354" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128717515[M 스포츠, 해외 공용 품번], 66128717499[기본형, 해외 공용 품번], 66128779005[디스플레이키, 해외 공용 품번], 66128717531[인디비주얼, 해외 공용 품번]</t>
         </is>
       </c>
       <c r="M354" s="11" t="inlineStr"/>
@@ -23988,7 +24459,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I355" s="11" t="inlineStr"/>
+      <c r="I355" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J355" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -23997,7 +24472,7 @@
       <c r="K355" s="11" t="inlineStr"/>
       <c r="L355" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128717515[M 스포츠, 해외 공용 품번], 66128717499[기본형, 해외 공용 품번], 66128779005[디스플레이키, 해외 공용 품번], 66128717531[인디비주얼, 해외 공용 품번]</t>
         </is>
       </c>
       <c r="M355" s="11" t="inlineStr"/>
@@ -25056,14 +25531,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I371" s="11" t="inlineStr"/>
+      <c r="I371" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J371" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
         </is>
       </c>
       <c r="K371" s="11" t="inlineStr"/>
-      <c r="L371" s="11" t="n"/>
+      <c r="L371" s="11" t="inlineStr">
+        <is>
+          <t>66128723582[M 스포츠], 66129254893[기본형], 66129254909[럭셔리 라인]</t>
+        </is>
+      </c>
       <c r="M371" s="11" t="inlineStr"/>
       <c r="N371" s="11" t="inlineStr">
         <is>
@@ -25184,14 +25667,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I373" s="11" t="inlineStr"/>
+      <c r="I373" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J373" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
         </is>
       </c>
       <c r="K373" s="11" t="inlineStr"/>
-      <c r="L373" s="11" t="inlineStr"/>
+      <c r="L373" s="11" t="inlineStr">
+        <is>
+          <t>66128723582[M 스포츠], 66129254893[기본형], 66129254909[럭셔리 라인]</t>
+        </is>
+      </c>
       <c r="M373" s="11" t="inlineStr"/>
       <c r="N373" s="17" t="inlineStr">
         <is>
@@ -25246,7 +25737,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I374" s="11" t="inlineStr"/>
+      <c r="I374" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J374" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -25255,7 +25750,7 @@
       <c r="K374" s="11" t="inlineStr"/>
       <c r="L374" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5662</t>
+          <t>FCC YGOHUF5662, 66128723582[M 스포츠], 66129254893[기본형], 66129254909[럭셔리 라인]</t>
         </is>
       </c>
       <c r="M374" s="11" t="inlineStr"/>
@@ -25312,7 +25807,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I375" s="11" t="inlineStr"/>
+      <c r="I375" s="11" t="inlineStr">
+        <is>
+          <t>51217268293[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J375" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -25321,7 +25820,7 @@
       <c r="K375" s="11" t="inlineStr"/>
       <c r="L375" s="11" t="inlineStr">
         <is>
-          <t>FCC YGOHUF5662</t>
+          <t>FCC YGOHUF5662, 66128723582[M 스포츠], 66129254893[기본형], 66129254909[럭셔리 라인]</t>
         </is>
       </c>
       <c r="M375" s="11" t="inlineStr"/>
@@ -25510,7 +26009,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I378" s="11" t="inlineStr"/>
+      <c r="I378" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J378" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -25519,7 +26022,7 @@
       <c r="K378" s="11" t="inlineStr"/>
       <c r="L378" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128717519[M 스포츠], 66128717503[기본형], 66128779004[디스플레이키], 66128717535[인디비주얼]</t>
         </is>
       </c>
       <c r="M378" s="11" t="inlineStr"/>
@@ -26509,7 +27012,7 @@
       <c r="K393" s="11" t="inlineStr"/>
       <c r="L393" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8FZV[3버튼]</t>
+          <t>FCC LX8FZV[3버튼], 66126955747[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M393" s="11" t="inlineStr"/>
@@ -26575,7 +27078,7 @@
       <c r="K394" s="11" t="inlineStr"/>
       <c r="L394" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8FZV</t>
+          <t>FCC LX8FZV, 66126955747[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M394" s="11" t="inlineStr"/>
@@ -26698,7 +27201,11 @@
           <t>막대키</t>
         </is>
       </c>
-      <c r="I396" s="11" t="inlineStr"/>
+      <c r="I396" s="11" t="inlineStr">
+        <is>
+          <t>51217127047[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J396" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -26707,7 +27214,7 @@
       <c r="K396" s="11" t="inlineStr"/>
       <c r="L396" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8FZV</t>
+          <t>FCC LX8FZV, 66126955747[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M396" s="11" t="inlineStr"/>
@@ -26764,7 +27271,11 @@
           <t>막대키</t>
         </is>
       </c>
-      <c r="I397" s="11" t="inlineStr"/>
+      <c r="I397" s="11" t="inlineStr">
+        <is>
+          <t>51217127047[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J397" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -26773,7 +27284,7 @@
       <c r="K397" s="11" t="inlineStr"/>
       <c r="L397" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8FZV</t>
+          <t>FCC LX8FZV, 66126955747[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M397" s="11" t="inlineStr"/>
@@ -26830,7 +27341,11 @@
           <t>막대키</t>
         </is>
       </c>
-      <c r="I398" s="11" t="inlineStr"/>
+      <c r="I398" s="11" t="inlineStr">
+        <is>
+          <t>51217127047[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J398" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -26839,7 +27354,7 @@
       <c r="K398" s="11" t="inlineStr"/>
       <c r="L398" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8FZV</t>
+          <t>FCC LX8FZV, 66126955747[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M398" s="11" t="inlineStr"/>
@@ -26896,7 +27411,11 @@
           <t>막대키</t>
         </is>
       </c>
-      <c r="I399" s="11" t="inlineStr"/>
+      <c r="I399" s="11" t="inlineStr">
+        <is>
+          <t>51217127047[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J399" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -26905,7 +27424,7 @@
       <c r="K399" s="11" t="inlineStr"/>
       <c r="L399" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8FZV</t>
+          <t>FCC LX8FZV, 66126955747[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M399" s="11" t="inlineStr"/>
@@ -26962,14 +27481,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I400" s="11" t="inlineStr"/>
+      <c r="I400" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J400" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
         </is>
       </c>
       <c r="K400" s="11" t="inlineStr"/>
-      <c r="L400" s="11" t="inlineStr"/>
+      <c r="L400" s="11" t="inlineStr">
+        <is>
+          <t>66126986584, 66129268487[컴포트액세스]</t>
+        </is>
+      </c>
       <c r="M400" s="11" t="inlineStr"/>
       <c r="N400" s="11" t="inlineStr">
         <is>
@@ -27288,14 +27815,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I405" s="11" t="inlineStr"/>
+      <c r="I405" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J405" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
         </is>
       </c>
       <c r="K405" s="11" t="inlineStr"/>
-      <c r="L405" s="11" t="inlineStr"/>
+      <c r="L405" s="11" t="inlineStr">
+        <is>
+          <t>66126986584, 66126986580[컴포트액세스]</t>
+        </is>
+      </c>
       <c r="M405" s="11" t="inlineStr"/>
       <c r="N405" s="11" t="inlineStr">
         <is>
@@ -27350,7 +27885,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I406" s="11" t="inlineStr"/>
+      <c r="I406" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J406" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
@@ -27359,7 +27898,7 @@
       <c r="K406" s="11" t="inlineStr"/>
       <c r="L406" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127</t>
+          <t>FCC KR55WK49127, 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M406" s="11" t="inlineStr"/>
@@ -27416,7 +27955,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I407" s="11" t="inlineStr"/>
+      <c r="I407" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J407" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
@@ -27425,7 +27968,7 @@
       <c r="K407" s="11" t="inlineStr"/>
       <c r="L407" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49123</t>
+          <t>FCC KR55WK49123, 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M407" s="11" t="inlineStr"/>
@@ -27482,7 +28025,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I408" s="11" t="inlineStr"/>
+      <c r="I408" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J408" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
@@ -27491,7 +28038,7 @@
       <c r="K408" s="11" t="inlineStr"/>
       <c r="L408" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49123, FCC KR55WK49127</t>
+          <t>FCC KR55WK49123, FCC KR55WK49127, 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M408" s="11" t="inlineStr"/>
@@ -27548,7 +28095,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I409" s="11" t="inlineStr"/>
+      <c r="I409" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J409" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -27614,7 +28165,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I410" s="11" t="inlineStr"/>
+      <c r="I410" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J410" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -27944,7 +28499,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I415" s="11" t="inlineStr"/>
+      <c r="I415" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J415" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -27953,7 +28512,7 @@
       <c r="K415" s="11" t="inlineStr"/>
       <c r="L415" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128708348, 66128708364[M 스포츠], 66128708340[기본형], 66129855654[디스플레이키], 66128708372[인디비주얼]</t>
         </is>
       </c>
       <c r="M415" s="11" t="inlineStr"/>
@@ -28010,7 +28569,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I416" s="11" t="inlineStr"/>
+      <c r="I416" s="11" t="inlineStr">
+        <is>
+          <t>51217444576[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J416" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -28019,7 +28582,7 @@
       <c r="K416" s="11" t="inlineStr"/>
       <c r="L416" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128708348, 66128708364[M 스포츠], 66128708340[기본형], 66129855654[디스플레이키], 66128708372[인디비주얼]</t>
         </is>
       </c>
       <c r="M416" s="11" t="inlineStr"/>
@@ -28608,7 +29171,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I425" s="11" t="inlineStr"/>
+      <c r="I425" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J425" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -28617,7 +29184,7 @@
       <c r="K425" s="11" t="inlineStr"/>
       <c r="L425" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID2A</t>
+          <t>FCC N5F-ID2A, 66126805997</t>
         </is>
       </c>
       <c r="M425" s="11" t="inlineStr"/>
@@ -28674,7 +29241,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I426" s="11" t="inlineStr"/>
+      <c r="I426" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J426" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -28683,7 +29254,7 @@
       <c r="K426" s="11" t="inlineStr"/>
       <c r="L426" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID2A, FCC NBGIDGNG1</t>
+          <t>FCC N5F-ID2A, FCC NBGIDGNG1, 66126805997</t>
         </is>
       </c>
       <c r="M426" s="11" t="inlineStr"/>
@@ -29198,7 +29769,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I434" s="11" t="n"/>
+      <c r="I434" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J434" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
@@ -29207,7 +29782,7 @@
       <c r="K434" s="11" t="n"/>
       <c r="L434" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127[3버튼]</t>
+          <t>FCC KR55WK49127[3버튼], 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M434" s="11" t="n"/>
@@ -29264,7 +29839,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I435" s="11" t="n"/>
+      <c r="I435" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J435" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
@@ -29273,7 +29852,7 @@
       <c r="K435" s="11" t="n"/>
       <c r="L435" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127[3버튼]</t>
+          <t>FCC KR55WK49127[3버튼], 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M435" s="11" t="n"/>
@@ -29330,7 +29909,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I436" s="11" t="inlineStr"/>
+      <c r="I436" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J436" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
@@ -29339,7 +29922,7 @@
       <c r="K436" s="11" t="inlineStr"/>
       <c r="L436" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127</t>
+          <t>FCC KR55WK49127, 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M436" s="11" t="inlineStr"/>
@@ -29396,7 +29979,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I437" s="11" t="inlineStr"/>
+      <c r="I437" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J437" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
@@ -29405,7 +29992,7 @@
       <c r="K437" s="11" t="inlineStr"/>
       <c r="L437" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49147[컴포트액세스], 926886-02[컴포트액세스]</t>
+          <t>FCC KR55WK49147[컴포트액세스], 926886-02[컴포트액세스], 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M437" s="11" t="inlineStr"/>
@@ -29462,7 +30049,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I438" s="11" t="inlineStr"/>
+      <c r="I438" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J438" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
@@ -29471,7 +30062,7 @@
       <c r="K438" s="11" t="inlineStr"/>
       <c r="L438" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49147, FCC KR55WK49127</t>
+          <t>FCC KR55WK49147, FCC KR55WK49127, 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M438" s="11" t="inlineStr"/>
@@ -29528,14 +30119,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I439" s="11" t="inlineStr"/>
+      <c r="I439" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J439" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
         </is>
       </c>
       <c r="K439" s="11" t="inlineStr"/>
-      <c r="L439" s="11" t="inlineStr"/>
+      <c r="L439" s="11" t="inlineStr">
+        <is>
+          <t>66126986584, 66126986580[컴포트액세스]</t>
+        </is>
+      </c>
       <c r="M439" s="11" t="inlineStr"/>
       <c r="N439" s="11" t="inlineStr">
         <is>
@@ -29590,7 +30189,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I440" s="11" t="inlineStr"/>
+      <c r="I440" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J440" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
@@ -29599,7 +30202,7 @@
       <c r="K440" s="11" t="inlineStr"/>
       <c r="L440" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127, FCC KR55WK49123</t>
+          <t>FCC KR55WK49127, FCC KR55WK49123, 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M440" s="11" t="inlineStr"/>
@@ -29656,7 +30259,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I441" s="11" t="inlineStr"/>
+      <c r="I441" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J441" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
@@ -29665,7 +30272,7 @@
       <c r="K441" s="11" t="inlineStr"/>
       <c r="L441" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127</t>
+          <t>FCC KR55WK49127, 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M441" s="11" t="inlineStr"/>
@@ -29920,7 +30527,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I445" s="11" t="inlineStr"/>
+      <c r="I445" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J445" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -29929,7 +30540,7 @@
       <c r="K445" s="11" t="inlineStr"/>
       <c r="L445" s="11" t="inlineStr">
         <is>
-          <t>FCC NBGIDGNG1</t>
+          <t>FCC NBGIDGNG1, 66126805997</t>
         </is>
       </c>
       <c r="M445" s="11" t="inlineStr"/>
@@ -29986,7 +30597,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I446" s="11" t="inlineStr"/>
+      <c r="I446" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J446" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -29995,7 +30610,7 @@
       <c r="K446" s="11" t="inlineStr"/>
       <c r="L446" s="11" t="inlineStr">
         <is>
-          <t>FCC NBGIDGNG1</t>
+          <t>FCC NBGIDGNG1, 66126805997</t>
         </is>
       </c>
       <c r="M446" s="11" t="inlineStr"/>
@@ -30052,7 +30667,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I447" s="11" t="inlineStr"/>
+      <c r="I447" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J447" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -30061,7 +30680,7 @@
       <c r="K447" s="11" t="inlineStr"/>
       <c r="L447" s="11" t="inlineStr">
         <is>
-          <t>FCC NBGIDGNG1</t>
+          <t>FCC NBGIDGNG1, 66126805997</t>
         </is>
       </c>
       <c r="M447" s="11" t="inlineStr"/>
@@ -30782,7 +31401,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I458" s="11" t="inlineStr"/>
+      <c r="I458" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J458" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -30791,7 +31414,7 @@
       <c r="K458" s="11" t="inlineStr"/>
       <c r="L458" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66126805997</t>
         </is>
       </c>
       <c r="M458" s="11" t="inlineStr"/>
@@ -30848,7 +31471,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I459" s="11" t="inlineStr"/>
+      <c r="I459" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J459" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -30857,7 +31484,7 @@
       <c r="K459" s="11" t="inlineStr"/>
       <c r="L459" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A, FCC NBGIDGNG1</t>
+          <t>FCC N5F-ID21A, FCC NBGIDGNG1, 66126805997</t>
         </is>
       </c>
       <c r="M459" s="11" t="inlineStr"/>
@@ -32199,7 +32826,11 @@
         </is>
       </c>
       <c r="K479" s="11" t="inlineStr"/>
-      <c r="L479" s="11" t="inlineStr"/>
+      <c r="L479" s="11" t="inlineStr">
+        <is>
+          <t>66126955747[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="M479" s="11" t="inlineStr"/>
       <c r="N479" s="11" t="inlineStr">
         <is>
@@ -32263,7 +32894,7 @@
       <c r="K480" s="11" t="inlineStr"/>
       <c r="L480" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8FZV</t>
+          <t>FCC LX8FZV, 66126955747[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M480" s="11" t="inlineStr"/>
@@ -32329,7 +32960,7 @@
       <c r="K481" s="11" t="inlineStr"/>
       <c r="L481" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8FZV</t>
+          <t>FCC LX8FZV, 66126955747[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M481" s="11" t="inlineStr"/>
@@ -32395,7 +33026,7 @@
       <c r="K482" s="11" t="inlineStr"/>
       <c r="L482" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8FZV</t>
+          <t>FCC LX8FZV, 66126955747[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M482" s="11" t="inlineStr"/>
@@ -32461,7 +33092,7 @@
       <c r="K483" s="11" t="inlineStr"/>
       <c r="L483" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8FZV</t>
+          <t>FCC LX8FZV, 66126955747[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M483" s="11" t="inlineStr"/>
@@ -32527,7 +33158,7 @@
       <c r="K484" s="11" t="inlineStr"/>
       <c r="L484" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8FZV</t>
+          <t>FCC LX8FZV, 66126955747[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M484" s="11" t="inlineStr"/>
@@ -32593,7 +33224,7 @@
       <c r="K485" s="11" t="inlineStr"/>
       <c r="L485" s="11" t="inlineStr">
         <is>
-          <t>FCC LX8FZV</t>
+          <t>FCC LX8FZV, 66126955747[해외 공용 품번]</t>
         </is>
       </c>
       <c r="M485" s="11" t="inlineStr"/>
@@ -32650,14 +33281,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I486" s="11" t="inlineStr"/>
+      <c r="I486" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J486" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
         </is>
       </c>
       <c r="K486" s="11" t="inlineStr"/>
-      <c r="L486" s="11" t="inlineStr"/>
+      <c r="L486" s="11" t="inlineStr">
+        <is>
+          <t>66126986584, 66126986580[컴포트액세스]</t>
+        </is>
+      </c>
       <c r="M486" s="11" t="inlineStr"/>
       <c r="N486" s="11" t="inlineStr">
         <is>
@@ -32712,7 +33351,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I487" s="11" t="inlineStr"/>
+      <c r="I487" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J487" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
@@ -32721,7 +33364,7 @@
       <c r="K487" s="11" t="inlineStr"/>
       <c r="L487" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127</t>
+          <t>FCC KR55WK49127, 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M487" s="11" t="inlineStr"/>
@@ -32778,7 +33421,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I488" s="11" t="inlineStr"/>
+      <c r="I488" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J488" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
@@ -32787,7 +33434,7 @@
       <c r="K488" s="11" t="inlineStr"/>
       <c r="L488" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49127</t>
+          <t>FCC KR55WK49127, 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M488" s="11" t="inlineStr"/>
@@ -32844,7 +33491,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I489" s="11" t="inlineStr"/>
+      <c r="I489" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J489" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
@@ -32853,7 +33504,7 @@
       <c r="K489" s="11" t="inlineStr"/>
       <c r="L489" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49147[컴포트액세스], FCC KR55WK49127</t>
+          <t>FCC KR55WK49147[컴포트액세스], FCC KR55WK49127, 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M489" s="11" t="inlineStr"/>
@@ -32910,7 +33561,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I490" s="11" t="inlineStr"/>
+      <c r="I490" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J490" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
@@ -32919,7 +33574,7 @@
       <c r="K490" s="11" t="inlineStr"/>
       <c r="L490" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49147, FCC KR55WK49127</t>
+          <t>FCC KR55WK49147, FCC KR55WK49127, 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M490" s="11" t="inlineStr"/>
@@ -32976,7 +33631,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I491" s="11" t="inlineStr"/>
+      <c r="I491" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J491" s="11" t="inlineStr">
         <is>
           <t>HU92[세대 기준]</t>
@@ -32985,7 +33644,7 @@
       <c r="K491" s="11" t="inlineStr"/>
       <c r="L491" s="11" t="inlineStr">
         <is>
-          <t>FCC KR55WK49147, FCC KR55WK49127</t>
+          <t>FCC KR55WK49147, FCC KR55WK49127, 66126986584, 66126986580[컴포트액세스]</t>
         </is>
       </c>
       <c r="M491" s="11" t="inlineStr"/>
@@ -33240,7 +33899,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I495" s="11" t="inlineStr"/>
+      <c r="I495" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J495" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -33249,7 +33912,7 @@
       <c r="K495" s="11" t="inlineStr"/>
       <c r="L495" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128708356[M 스포츠], 66128708340[기본형], 66128708372[인디비주얼]</t>
         </is>
       </c>
       <c r="M495" s="11" t="inlineStr"/>
@@ -33306,7 +33969,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I496" s="11" t="inlineStr"/>
+      <c r="I496" s="11" t="inlineStr">
+        <is>
+          <t>51217409076[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J496" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -33315,7 +33982,7 @@
       <c r="K496" s="11" t="inlineStr"/>
       <c r="L496" s="11" t="inlineStr">
         <is>
-          <t>FCC N5F-ID21A</t>
+          <t>FCC N5F-ID21A, 66128708356[M 스포츠], 66128708340[기본형], 66128708372[인디비주얼]</t>
         </is>
       </c>
       <c r="M496" s="11" t="inlineStr"/>
@@ -34098,7 +34765,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I508" s="11" t="inlineStr"/>
+      <c r="I508" s="11" t="inlineStr">
+        <is>
+          <t>51217393289[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J508" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -34107,7 +34778,7 @@
       <c r="K508" s="11" t="inlineStr"/>
       <c r="L508" s="11" t="inlineStr">
         <is>
-          <t>FCC NBGIDGNG1</t>
+          <t>FCC NBGIDGNG1, 66128728010</t>
         </is>
       </c>
       <c r="M508" s="11" t="inlineStr"/>
@@ -34164,7 +34835,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I509" s="11" t="inlineStr"/>
+      <c r="I509" s="11" t="inlineStr">
+        <is>
+          <t>51217393289[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J509" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -34173,7 +34848,7 @@
       <c r="K509" s="11" t="inlineStr"/>
       <c r="L509" s="11" t="inlineStr">
         <is>
-          <t>FCC NBGIDGNG1</t>
+          <t>FCC NBGIDGNG1, 66128728010</t>
         </is>
       </c>
       <c r="M509" s="11" t="inlineStr"/>
@@ -34296,7 +34971,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I511" s="11" t="inlineStr"/>
+      <c r="I511" s="11" t="inlineStr">
+        <is>
+          <t>51217393289[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J511" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -34305,7 +34984,7 @@
       <c r="K511" s="11" t="inlineStr"/>
       <c r="L511" s="11" t="inlineStr">
         <is>
-          <t>FCC NBGIDGNG1[추정]</t>
+          <t>FCC NBGIDGNG1[추정], 66126805981</t>
         </is>
       </c>
       <c r="M511" s="11" t="inlineStr"/>
@@ -34494,7 +35173,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I514" s="11" t="inlineStr"/>
+      <c r="I514" s="11" t="inlineStr">
+        <is>
+          <t>51217393289[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J514" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -34503,7 +35186,7 @@
       <c r="K514" s="11" t="inlineStr"/>
       <c r="L514" s="11" t="inlineStr">
         <is>
-          <t>FCC NBGIDGNG1</t>
+          <t>FCC NBGIDGNG1, 66126805981</t>
         </is>
       </c>
       <c r="M514" s="11" t="inlineStr"/>
@@ -34626,7 +35309,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I516" s="11" t="inlineStr"/>
+      <c r="I516" s="11" t="inlineStr">
+        <is>
+          <t>51217393289[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J516" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -34635,7 +35322,7 @@
       <c r="K516" s="11" t="inlineStr"/>
       <c r="L516" s="11" t="inlineStr">
         <is>
-          <t>FCC NBGIDGNG1</t>
+          <t>FCC NBGIDGNG1, 66128728013</t>
         </is>
       </c>
       <c r="M516" s="11" t="inlineStr"/>
@@ -34692,7 +35379,11 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I517" s="11" t="inlineStr"/>
+      <c r="I517" s="11" t="inlineStr">
+        <is>
+          <t>51217393289[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J517" s="11" t="inlineStr">
         <is>
           <t>HU100R[세대 기준]</t>
@@ -34701,7 +35392,7 @@
       <c r="K517" s="11" t="inlineStr"/>
       <c r="L517" s="11" t="inlineStr">
         <is>
-          <t>FCC NBGIDGNG1</t>
+          <t>FCC NBGIDGNG1, 66128728013</t>
         </is>
       </c>
       <c r="M517" s="11" t="inlineStr"/>
@@ -35934,14 +36625,22 @@
           <t>스마트키</t>
         </is>
       </c>
-      <c r="I536" s="11" t="inlineStr"/>
+      <c r="I536" s="11" t="inlineStr">
+        <is>
+          <t>51217139710[해외 공용 품번]</t>
+        </is>
+      </c>
       <c r="J536" s="11" t="inlineStr">
         <is>
           <t>HU92</t>
         </is>
       </c>
       <c r="K536" s="11" t="inlineStr"/>
-      <c r="L536" s="11" t="n"/>
+      <c r="L536" s="11" t="inlineStr">
+        <is>
+          <t>66126986584</t>
+        </is>
+      </c>
       <c r="M536" s="11" t="inlineStr"/>
       <c r="N536" s="11" t="inlineStr">
         <is>
@@ -35967,408 +36666,415 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A61"/>
+  <dimension ref="A1:A62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>이 표는 락스미스(자동차 키 제작/프로그래밍) 참고용입니다.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="21" t="inlineStr"/>
+      <c r="A2" s="22" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>※ 구성</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>- 맨 앞 '브랜드' 컬럼에 브랜드명을 적었습니다(검색 프로그램에서 '기아 K5'처럼 브랜드와 모델명을 함께 검색 가능).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>- '키종류'는 그 연식에 나온 키 형태(막대키·폴딩키·스마트키·카드키)를 모두 적었습니다. 트림별로 다른 경우 함께 적었습니다(예: 폴딩키,스마트키).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>- 키 부품번호는 국내 사양(433/434MHz)만 적었습니다. 미국(315MHz)·유럽(868MHz) 사양 키는 뺐습니다.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>- '비고'에는 주황색·빨간색 칸의 이유만 적었습니다.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>- 컬럼은 '기아_트랜스폰더_칩코드_DBnew.xlsx'와 동일합니다. 모델마다 연식별로 한 행씩, 2000년식부터 기록했습니다(1990년대 출시 모델도 2000년식부터).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>- 연식이 '현재'인 모델은 2026년식까지, 단종 모델의 마지막 연식은 '2012(단종)' 형식으로 표기했습니다.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>- '이모빌라이저 시스템'은 차량 쪽 모듈(EWS3/EWS4, CAS1~CAS4+, FEM, BDC/BDC2/BDC3, BCP)을 적었습니다.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>- '스마트키(부품번호)'에는 BMW 순정 부품번호(66 12 …, 9xxxxxx-xx 등)와 FCC ID(KR55WK…, YGOHUF…, N5F-ID21A, IYZBK1 등)를 함께 적었습니다. CAS1~CAS3의 삽입식 리모컨키도 이 칸에 적고 괄호로 구분했습니다.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>- '키블레이드(부품번호)'는 해당 연식 검색 결과에 직접 나온 경우에만 적었고, 나오지 않은 칸은 공란입니다(기아 파일 규칙과 동일). 카드키·폴딩키는 BMW에 해당 형태가 없어 비워 두었습니다(E65 CAS1 슬롯형 키는 스마트키 칸에 기재).</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>- '키블레이드(키웨이)'에 '(세대 기준)'이 붙은 칸은 그 연식 검색에서 키웨이가 직접 확인되지 않아 같은 세대 기준으로 적은 값입니다. '(추정)'은 신형 차종에서 근거가 약한 값입니다.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>- 'XT27A/A66·XT27B·XT57B 호환'은 칩 종류 기준으로 기아 파일의 표기 규칙을 그대로 따랐습니다: ID46·ID44 → O/O/O, ID49(Hitag Pro) → X/△/O, ID46·ID49 병기 → △/△/O. (근거: Xhorse 슈퍼칩 비교 — XT27A는 ID49 미지원, XT27B·XT57B는 ID49 지원 표기) 실제 차량 적용 전 장비로 재확인하세요.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>- 출처 칸의 사이트명은 해당 연식 검색에서 근거로 쓴 페이지입니다. 이 환경에서는 부품몰 원문을 직접 열 수 없어 검색 결과 요약을 근거로 했습니다.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr"/>
+      <c r="A16" s="22" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="22" t="inlineStr">
         <is>
           <t>※ 색상</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>- 빨간색: 확인 불가/확인 필요 — 절대 그대로 신뢰해서 작업하지 마세요.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="22" t="inlineStr">
         <is>
           <t>- 주황색: 출처가 서로 상충하거나 원문으로 직접 확인되지 않은 경우 — 작업 전 VIN/실물 모듈로 재확인.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="21" t="inlineStr">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>- 전환기(EWS3→EWS4, CAS1→CAS2, CAS2→CAS3, CAS3→CAS3+, CAS4→CAS4+, BDC2→BDC3)는 색 표시 없이 이모빌라이저 칸에 전환 전·후를 함께 적었습니다(예: CAS3(2008 중반 이전 생산) / CAS3+(2008 중반 이후 생산)).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="inlineStr"/>
+      <c r="A21" s="22" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>※ 조사하며 확인된 주요 사항</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>- CAS4/CAS4+ 키의 칩은 ID49(PCF7953)입니다(Hitag Pro 계열, 이전 초안의 'Hitag2' 표기는 오류였음). 일부 판매처는 이 칩을 'EWS5'로 부르지만 이모빌라이저 이름(EWS)과 헷갈려 쓰지 않았습니다.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="22" t="inlineStr">
         <is>
           <t>- CAS4+ 도입 시점은 자료마다 다릅니다(2012 중반 이후 생산분 vs 2013년 F10부터) — 2012년식은 주황색.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="21" t="inlineStr">
+      <c r="A25" s="22" t="inlineStr">
         <is>
           <t>- [이모빌라이저 재검증] F20/F22/F30/F32/F80/F82/F87은 LCI 이후에도 FEM(딜러 부품 FEM 61355A7FB57 등) — BDC가 아닙니다. F15/F16/F85/F86/F45/F48/F39/i3/i8은 BDC.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="22" t="inlineStr">
         <is>
           <t>- BDC2(BDC_G11): G11/G12(~2019.2), G30/G31/G32/F90(~2020.6), G01/G02/F97/F98(~2021.7), G08(~2021.8). 이후 생산분은 BDC3.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="21" t="inlineStr">
+      <c r="A27" s="22" t="inlineStr">
         <is>
           <t>- BDC3(BDC_G05): G05/G06/G07/G20/G15/G29/F40/F44/G42/G22/G80/G82/G87/F95/F96은 출시부터 BDC3.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="A28" s="22" t="inlineStr">
         <is>
           <t>- BCP: i7/7시리즈 G70·iX(딜러 부품 'Control u.basic computing platform (BCP)' 61355A9A210), U06/U10/U11, G45. G60/i5/G90은 BDC3·BCP 자료 상충(주황색).</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="21" t="inlineStr">
+      <c r="A29" s="22" t="inlineStr">
         <is>
           <t>- BDC2 키: N5F-ID21A(9367401-01), 2022년 이후 순정 키: IYZBK1.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="21" t="inlineStr">
+      <c r="A30" s="22" t="inlineStr">
         <is>
           <t>- U섀시(U06/U10/U11)는 BCP 이모빌라이저 + UWB 키(NCF2951/Hitag Pro/ID49, FCC IYZBK1).</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="21" t="inlineStr">
+      <c r="A31" s="22" t="inlineStr">
         <is>
           <t>- E65는 2005 LCI 전 CAS1, 이후 CAS2. E60/E61/E63은 2007.3 LCI 전 CAS2, 이후 CAS3. E83은 2006 중 EWS3→EWS4.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="21" t="n"/>
+      <c r="A32" s="22" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="21" t="inlineStr">
+      <c r="A33" s="22" t="inlineStr">
         <is>
           <t>※ 표기 규칙 (칩코드·부품번호·키웨이·이모빌라이저 칸 공통)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="21" t="inlineStr">
+      <c r="A34" s="22" t="inlineStr">
         <is>
           <t>- 한 칸에 값이 여러 개면 ', '(쉼표)로만 구분합니다. '/', '·', '또는'은 쓰지 않고, 줄임(예: 4F0837220M/T, 5WK49145~49147)도 모두 풀어서 따로 적었습니다.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="21" t="inlineStr">
+      <c r="A35" s="22" t="inlineStr">
         <is>
           <t>- ( ) 안에는 부품번호만 적습니다. 칩코드 'ID49(PCF7953)' = ID49 칩, 칩 부품번호 PCF7953. 이모빌라이저 'SKM(87570-36010)' = SKM 모듈, 품번 87570-36010. 칩 부품번호를 모르면 'ID46'처럼 ID만 적었습니다.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="21" t="inlineStr">
+      <c r="A36" s="22" t="inlineStr">
         <is>
           <t>- [ ] 안에는 그 값이 적용되는 조건을 적습니다(키 종류·버튼 수·옵션·생산 시기·차종 코드). 예: ID46(PCF7936)[폴딩키], ID46(PCF7952A)[스마트키] → 폴딩키는 PCF7936, 스마트키는 PCF7952A.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="21" t="inlineStr">
+      <c r="A37" s="22" t="inlineStr">
         <is>
           <t>- [추정] = 추정값, [일부 자료] = 일부 자료에만 나오는 값, [자료 상충] = 자료마다 달라 둘 중 무엇인지 미확정, [해외 공용 품번] = 해외 공용 품번(국내 순정 품번 미확인).</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="21" t="inlineStr">
+      <c r="A38" s="22" t="inlineStr">
         <is>
           <t>- 부품번호 칸에는 부품번호만 적습니다. 'FCC ' = 미국 FCC 인증번호(키 모델 식별용), 'KC ' = 한국 전파인증번호. 순정(제조사) 부품번호만 적고 애프터마켓 호환품 번호는 넣지 않았습니다. 설명·판매처·주파수(모두 국내 433/434MHz)는 적지 않았고, 부품번호가 없으면 공란입니다.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="21" t="inlineStr">
+      <c r="A39" s="22" t="inlineStr">
         <is>
           <t>- Hitag2·Hitag Pro·Megamos·DST80 같은 칩 방식 이름은 ID 코드와 같은 뜻이라 칸에 따로 적지 않았습니다(아래 표).</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="21" t="n"/>
+      <c r="A40" s="22" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="21" t="inlineStr">
+      <c r="A41" s="22" t="inlineStr">
         <is>
           <t>※ 칩 ID 코드 뜻</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="21" t="inlineStr">
+      <c r="A42" s="22" t="inlineStr">
         <is>
           <t>- ID13: Megamos 13(고정 코드)  |  ID44: Philips Crypto(PCF7935, BMW EWS 구형)  |  ID48: Megamos Crypto</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="21" t="inlineStr">
+      <c r="A43" s="22" t="inlineStr">
         <is>
           <t>- ID46: Philips Hitag2 계열(PCF7936·PCF7941·PCF7945·PCF7952 등). [Extended] = Hitag2 Extended, [Circle Plus] = GM Circle Plus</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="21" t="inlineStr">
+      <c r="A44" s="22" t="inlineStr">
         <is>
           <t>- ID47: NXP Hitag3(NCF2951·NCF2952·NCF2971·PCF7938 등)  |  ID49: NXP Hitag Pro(PCF7953P·NCF2951·NCF295X 등)  |  ID4A: NXP Hitag AES(NCF29A1M·PCF7953M·PCF7961M 등)</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="21" t="inlineStr">
+      <c r="A45" s="22" t="inlineStr">
         <is>
           <t>- ID60: Texas 4D60(40bit)  |  4D60x80: Texas 4D60 80bit(DST80 계열)  |  ID70: Texas 4D70  |  ID6E-MA: Texas DST80(현대·기아 표기)</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="21" t="inlineStr">
+      <c r="A46" s="22" t="inlineStr">
         <is>
           <t>- ID6A·ID8A: Texas Crypto AES(DST-AES)  |  ID75: Texas AES(판매처 표기)  |  ID88: Megamos AES(VW·아우디 MQB)  |  ID8E: 아우디 8E Crypto(Sokymat 8E)</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="21" t="inlineStr">
+      <c r="A47" s="22" t="inlineStr">
         <is>
           <t>- FBS3·FBS4: 벤츠 NEC 프로세서 키(ID 칩이 아님)  |  MLB 전용 칩·MLB evo 전용 칩: 아우디 MLB 플랫폼 전용 키 칩</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="21" t="inlineStr">
+      <c r="A48" s="22" t="inlineStr">
         <is>
           <t>- 확인 불가 = 자료로 확인하지 못함  |  해당 없음 = 이모빌라이저 미적용</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="21" t="n"/>
+      <c r="A49" s="22" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="21" t="inlineStr">
+      <c r="A50" s="22" t="inlineStr">
         <is>
           <t>※ 재조사로 확인한 근거 (색을 지운 행)</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="21" t="inlineStr">
+      <c r="A51" s="22" t="inlineStr">
         <is>
           <t>- BMW G60·i5·M5·X7 LCI: 키 프로그래머 업체(Autel·KeyDIY·Xhorse)가 G섀시(G30/G31/G60 2020.7~)를 BDC3, U섀시를 BCP로 구분 — G60은 BDC3 Add Key 대상으로 명시(obdii365·obd2.ltd)</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="21" t="inlineStr">
+      <c r="A52" s="22" t="inlineStr">
         <is>
           <t>- BMW XM G09: IYZBK1 키(X5·X6·X7·XM 공용, UWB) — G섀시 BDC3 키 복사·추가 대상(Xhorse G chassis BDC3)</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="21" t="inlineStr">
+      <c r="A53" s="22" t="inlineStr">
         <is>
           <t>- BMW X4 F26 2016: 순정 CAS4+ 키 칩은 PCF7953(ID49) — PCF7945P는 "CAS4 modified type" 애프터마켓 키 칩(mk3·vvdi)이라 뺌</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="21" t="inlineStr">
+      <c r="A54" s="22" t="inlineStr">
         <is>
           <t>- BMW E90 CAS3+: 순정 키 칩 PCF7945·PCF7943·PCF7944 모두 ID46(Hitag2) 계열로 병존(bimmerfest·keyecu) — 자료 상충 아님</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="21" t="inlineStr">
+      <c r="A55" s="22" t="inlineStr">
         <is>
           <t>- BMW X3 G45: Lonsdor K518 PRO "2025 BMW X3 UWB에 BCP 키 추가" 절차(U섀시 BCP) 확인 — 이모빌라이저 BCP 확정</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="21" t="inlineStr">
+      <c r="A56" s="22" t="inlineStr">
         <is>
           <t>- BMW X3 F25 2013: CAS4+ 순정 키 칩 PCF7953(ID49) — 같이 적혀 있던 PCF7945P는 중국산 CAS4 호환 키 칩(mr-key·tlkeys 판매품)이라 뺌(X4 F26과 같은 판단)</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="21" t="n"/>
+      <c r="A57" s="22" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="21" t="inlineStr">
+      <c r="A58" s="22" t="inlineStr">
         <is>
           <t>※ 행 구분 규칙</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="21" t="inlineStr">
+      <c r="A59" s="22" t="inlineStr">
         <is>
           <t>- 연식 중간에 칩·이모빌라이저·키가 바뀐 해는 바뀌기 전·후를 따로 행으로 나눔. 세대가 바뀌면 세대별 모델명으로 1행씩, 같은 세대 안의 변경(부분변경·생산 시기·키 변경)은 같은 모델명으로 나누고 칸 안의 [생산 시기]·[세대] 표기로 구분</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="21" t="inlineStr">
+      <c r="A60" s="22" t="inlineStr">
         <is>
           <t>- 같은 연식·모델에 행이 2개인데 칸에 시기 표기가 없으면(예: 벤츠 FBS3 행과 FBS4 행) 전환 시점 자료가 없는 것 — 주황색, 비고의 방법(VIN 등)으로 확인</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="21" t="inlineStr">
+      <c r="A61" s="22" t="inlineStr">
         <is>
           <t>- BMW 순정 부품번호(애프터마켓 대체): 비상키 51215A4FBE5 = F40·F44·G20·G22·G26·G42·G80·G82 등 인서트 키(recambiosyaccesoriosbmw), 51215A65D30 = U06·U10·U11·G60·G70·I20 등 인서트 키, 리모컨 66125A473F4(M 스포츠, ECE+RoW+US) = F40·F44·F9x·G01·G42·G87·G80·G82(hubauer·딜러몰), 66125A47402(기본, ECE+RoW) = G01·G02·G08·G11·G12·G30(schmiedmann), 66125A56076(기본, ECE+RoW) = F15·F16·F39·F45·F46·F48(hubauer), 66128708328(기본, ECE+RoW+US) = F40·G29(hubauer), 66125B3E8E1(M, ECE+RoW) = G60·G70·I20·U06·U10·U11 등, 66129362173 = i3 I01 434MHz(66126805980 대체), 51217127047 = X3 E83 도어·점화 키 — 한국 사양(KO) 번호 적용 차종은 미확인이라 [해외 공용 품번]</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="22" t="inlineStr">
+        <is>
+          <t>- BMW ETK(etkbmw.cc, 카탈로그 03.2019) 키 부품: 한국 사양(L802A National version Korea) 조건 번호가 있으면 그대로(태그 없음), 없으면 국가 제한 없는 번호를 [해외 공용 품번]으로 기재. 한국 사양 CAS 리모컨은 315MHz 저출력 전용 품번(예: 66126986584 = E60·E63·E70·E71·E84·E89 등, 2005.9 이전 E60·E63은 66126933076), E83 X3 한국 사양은 적외선 리모컨 51218374933도 등재. 트림 태그(기본형·스포츠 라인·럭셔리 라인·M 스포츠 등)는 ETK 키 디자인 구분, M 모델은 M·M 스포츠·디스플레이키·컴포트액세스만. 2021년식 이후와 E38·E39는 카탈로그 범위 밖이라 미기재</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BMW guide: clarify Korean key frequency by generation
E-series (CAS2/CAS3) Korean-spec keys are listed in ETK only as 315MHz low power;
the 434MHz keys carry a 'without National version Korea' condition. F/G/I-series
Korean-spec keys are 434MHz.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GdWs29tcwv2723Uq4P5rH7
</commit_message>
<xml_diff>
--- a/BMW_코리아_출시모델.xlsx
+++ b/BMW_코리아_출시모델.xlsx
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -188,6 +188,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -36673,408 +36676,408 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="22" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>이 표는 락스미스(자동차 키 제작/프로그래밍) 참고용입니다.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="inlineStr"/>
+      <c r="A2" s="23" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="22" t="inlineStr">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>※ 구성</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>- 맨 앞 '브랜드' 컬럼에 브랜드명을 적었습니다(검색 프로그램에서 '기아 K5'처럼 브랜드와 모델명을 함께 검색 가능).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="22" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>- '키종류'는 그 연식에 나온 키 형태(막대키·폴딩키·스마트키·카드키)를 모두 적었습니다. 트림별로 다른 경우 함께 적었습니다(예: 폴딩키,스마트키).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>- 키 부품번호는 국내 사양(433/434MHz)만 적었습니다. 미국(315MHz)·유럽(868MHz) 사양 키는 뺐습니다.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>- '비고'에는 주황색·빨간색 칸의 이유만 적었습니다.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>- 컬럼은 '기아_트랜스폰더_칩코드_DBnew.xlsx'와 동일합니다. 모델마다 연식별로 한 행씩, 2000년식부터 기록했습니다(1990년대 출시 모델도 2000년식부터).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>- 연식이 '현재'인 모델은 2026년식까지, 단종 모델의 마지막 연식은 '2012(단종)' 형식으로 표기했습니다.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>- '이모빌라이저 시스템'은 차량 쪽 모듈(EWS3/EWS4, CAS1~CAS4+, FEM, BDC/BDC2/BDC3, BCP)을 적었습니다.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="22" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>- '스마트키(부품번호)'에는 BMW 순정 부품번호(66 12 …, 9xxxxxx-xx 등)와 FCC ID(KR55WK…, YGOHUF…, N5F-ID21A, IYZBK1 등)를 함께 적었습니다. CAS1~CAS3의 삽입식 리모컨키도 이 칸에 적고 괄호로 구분했습니다.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>- '키블레이드(부품번호)'는 해당 연식 검색 결과에 직접 나온 경우에만 적었고, 나오지 않은 칸은 공란입니다(기아 파일 규칙과 동일). 카드키·폴딩키는 BMW에 해당 형태가 없어 비워 두었습니다(E65 CAS1 슬롯형 키는 스마트키 칸에 기재).</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>- '키블레이드(키웨이)'에 '(세대 기준)'이 붙은 칸은 그 연식 검색에서 키웨이가 직접 확인되지 않아 같은 세대 기준으로 적은 값입니다. '(추정)'은 신형 차종에서 근거가 약한 값입니다.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="22" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>- 'XT27A/A66·XT27B·XT57B 호환'은 칩 종류 기준으로 기아 파일의 표기 규칙을 그대로 따랐습니다: ID46·ID44 → O/O/O, ID49(Hitag Pro) → X/△/O, ID46·ID49 병기 → △/△/O. (근거: Xhorse 슈퍼칩 비교 — XT27A는 ID49 미지원, XT27B·XT57B는 ID49 지원 표기) 실제 차량 적용 전 장비로 재확인하세요.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="22" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>- 출처 칸의 사이트명은 해당 연식 검색에서 근거로 쓴 페이지입니다. 이 환경에서는 부품몰 원문을 직접 열 수 없어 검색 결과 요약을 근거로 했습니다.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="inlineStr"/>
+      <c r="A16" s="23" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>※ 색상</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="22" t="inlineStr">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>- 빨간색: 확인 불가/확인 필요 — 절대 그대로 신뢰해서 작업하지 마세요.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="22" t="inlineStr">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>- 주황색: 출처가 서로 상충하거나 원문으로 직접 확인되지 않은 경우 — 작업 전 VIN/실물 모듈로 재확인.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="22" t="inlineStr">
+      <c r="A20" s="23" t="inlineStr">
         <is>
           <t>- 전환기(EWS3→EWS4, CAS1→CAS2, CAS2→CAS3, CAS3→CAS3+, CAS4→CAS4+, BDC2→BDC3)는 색 표시 없이 이모빌라이저 칸에 전환 전·후를 함께 적었습니다(예: CAS3(2008 중반 이전 생산) / CAS3+(2008 중반 이후 생산)).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="22" t="inlineStr"/>
+      <c r="A21" s="23" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="22" t="inlineStr">
+      <c r="A22" s="23" t="inlineStr">
         <is>
           <t>※ 조사하며 확인된 주요 사항</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="22" t="inlineStr">
+      <c r="A23" s="23" t="inlineStr">
         <is>
           <t>- CAS4/CAS4+ 키의 칩은 ID49(PCF7953)입니다(Hitag Pro 계열, 이전 초안의 'Hitag2' 표기는 오류였음). 일부 판매처는 이 칩을 'EWS5'로 부르지만 이모빌라이저 이름(EWS)과 헷갈려 쓰지 않았습니다.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="22" t="inlineStr">
+      <c r="A24" s="23" t="inlineStr">
         <is>
           <t>- CAS4+ 도입 시점은 자료마다 다릅니다(2012 중반 이후 생산분 vs 2013년 F10부터) — 2012년식은 주황색.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="22" t="inlineStr">
+      <c r="A25" s="23" t="inlineStr">
         <is>
           <t>- [이모빌라이저 재검증] F20/F22/F30/F32/F80/F82/F87은 LCI 이후에도 FEM(딜러 부품 FEM 61355A7FB57 등) — BDC가 아닙니다. F15/F16/F85/F86/F45/F48/F39/i3/i8은 BDC.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="22" t="inlineStr">
+      <c r="A26" s="23" t="inlineStr">
         <is>
           <t>- BDC2(BDC_G11): G11/G12(~2019.2), G30/G31/G32/F90(~2020.6), G01/G02/F97/F98(~2021.7), G08(~2021.8). 이후 생산분은 BDC3.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="22" t="inlineStr">
+      <c r="A27" s="23" t="inlineStr">
         <is>
           <t>- BDC3(BDC_G05): G05/G06/G07/G20/G15/G29/F40/F44/G42/G22/G80/G82/G87/F95/F96은 출시부터 BDC3.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="22" t="inlineStr">
+      <c r="A28" s="23" t="inlineStr">
         <is>
           <t>- BCP: i7/7시리즈 G70·iX(딜러 부품 'Control u.basic computing platform (BCP)' 61355A9A210), U06/U10/U11, G45. G60/i5/G90은 BDC3·BCP 자료 상충(주황색).</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="22" t="inlineStr">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>- BDC2 키: N5F-ID21A(9367401-01), 2022년 이후 순정 키: IYZBK1.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="22" t="inlineStr">
+      <c r="A30" s="23" t="inlineStr">
         <is>
           <t>- U섀시(U06/U10/U11)는 BCP 이모빌라이저 + UWB 키(NCF2951/Hitag Pro/ID49, FCC IYZBK1).</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="22" t="inlineStr">
+      <c r="A31" s="23" t="inlineStr">
         <is>
           <t>- E65는 2005 LCI 전 CAS1, 이후 CAS2. E60/E61/E63은 2007.3 LCI 전 CAS2, 이후 CAS3. E83은 2006 중 EWS3→EWS4.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="22" t="n"/>
+      <c r="A32" s="23" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="22" t="inlineStr">
+      <c r="A33" s="23" t="inlineStr">
         <is>
           <t>※ 표기 규칙 (칩코드·부품번호·키웨이·이모빌라이저 칸 공통)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="22" t="inlineStr">
+      <c r="A34" s="23" t="inlineStr">
         <is>
           <t>- 한 칸에 값이 여러 개면 ', '(쉼표)로만 구분합니다. '/', '·', '또는'은 쓰지 않고, 줄임(예: 4F0837220M/T, 5WK49145~49147)도 모두 풀어서 따로 적었습니다.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="22" t="inlineStr">
+      <c r="A35" s="23" t="inlineStr">
         <is>
           <t>- ( ) 안에는 부품번호만 적습니다. 칩코드 'ID49(PCF7953)' = ID49 칩, 칩 부품번호 PCF7953. 이모빌라이저 'SKM(87570-36010)' = SKM 모듈, 품번 87570-36010. 칩 부품번호를 모르면 'ID46'처럼 ID만 적었습니다.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="22" t="inlineStr">
+      <c r="A36" s="23" t="inlineStr">
         <is>
           <t>- [ ] 안에는 그 값이 적용되는 조건을 적습니다(키 종류·버튼 수·옵션·생산 시기·차종 코드). 예: ID46(PCF7936)[폴딩키], ID46(PCF7952A)[스마트키] → 폴딩키는 PCF7936, 스마트키는 PCF7952A.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="22" t="inlineStr">
+      <c r="A37" s="23" t="inlineStr">
         <is>
           <t>- [추정] = 추정값, [일부 자료] = 일부 자료에만 나오는 값, [자료 상충] = 자료마다 달라 둘 중 무엇인지 미확정, [해외 공용 품번] = 해외 공용 품번(국내 순정 품번 미확인).</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="22" t="inlineStr">
+      <c r="A38" s="23" t="inlineStr">
         <is>
           <t>- 부품번호 칸에는 부품번호만 적습니다. 'FCC ' = 미국 FCC 인증번호(키 모델 식별용), 'KC ' = 한국 전파인증번호. 순정(제조사) 부품번호만 적고 애프터마켓 호환품 번호는 넣지 않았습니다. 설명·판매처·주파수(모두 국내 433/434MHz)는 적지 않았고, 부품번호가 없으면 공란입니다.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="22" t="inlineStr">
+      <c r="A39" s="23" t="inlineStr">
         <is>
           <t>- Hitag2·Hitag Pro·Megamos·DST80 같은 칩 방식 이름은 ID 코드와 같은 뜻이라 칸에 따로 적지 않았습니다(아래 표).</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="22" t="n"/>
+      <c r="A40" s="23" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="22" t="inlineStr">
+      <c r="A41" s="23" t="inlineStr">
         <is>
           <t>※ 칩 ID 코드 뜻</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="22" t="inlineStr">
+      <c r="A42" s="23" t="inlineStr">
         <is>
           <t>- ID13: Megamos 13(고정 코드)  |  ID44: Philips Crypto(PCF7935, BMW EWS 구형)  |  ID48: Megamos Crypto</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="22" t="inlineStr">
+      <c r="A43" s="23" t="inlineStr">
         <is>
           <t>- ID46: Philips Hitag2 계열(PCF7936·PCF7941·PCF7945·PCF7952 등). [Extended] = Hitag2 Extended, [Circle Plus] = GM Circle Plus</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="22" t="inlineStr">
+      <c r="A44" s="23" t="inlineStr">
         <is>
           <t>- ID47: NXP Hitag3(NCF2951·NCF2952·NCF2971·PCF7938 등)  |  ID49: NXP Hitag Pro(PCF7953P·NCF2951·NCF295X 등)  |  ID4A: NXP Hitag AES(NCF29A1M·PCF7953M·PCF7961M 등)</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="22" t="inlineStr">
+      <c r="A45" s="23" t="inlineStr">
         <is>
           <t>- ID60: Texas 4D60(40bit)  |  4D60x80: Texas 4D60 80bit(DST80 계열)  |  ID70: Texas 4D70  |  ID6E-MA: Texas DST80(현대·기아 표기)</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="22" t="inlineStr">
+      <c r="A46" s="23" t="inlineStr">
         <is>
           <t>- ID6A·ID8A: Texas Crypto AES(DST-AES)  |  ID75: Texas AES(판매처 표기)  |  ID88: Megamos AES(VW·아우디 MQB)  |  ID8E: 아우디 8E Crypto(Sokymat 8E)</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="22" t="inlineStr">
+      <c r="A47" s="23" t="inlineStr">
         <is>
           <t>- FBS3·FBS4: 벤츠 NEC 프로세서 키(ID 칩이 아님)  |  MLB 전용 칩·MLB evo 전용 칩: 아우디 MLB 플랫폼 전용 키 칩</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="22" t="inlineStr">
+      <c r="A48" s="23" t="inlineStr">
         <is>
           <t>- 확인 불가 = 자료로 확인하지 못함  |  해당 없음 = 이모빌라이저 미적용</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="22" t="n"/>
+      <c r="A49" s="23" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="22" t="inlineStr">
+      <c r="A50" s="23" t="inlineStr">
         <is>
           <t>※ 재조사로 확인한 근거 (색을 지운 행)</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="22" t="inlineStr">
+      <c r="A51" s="23" t="inlineStr">
         <is>
           <t>- BMW G60·i5·M5·X7 LCI: 키 프로그래머 업체(Autel·KeyDIY·Xhorse)가 G섀시(G30/G31/G60 2020.7~)를 BDC3, U섀시를 BCP로 구분 — G60은 BDC3 Add Key 대상으로 명시(obdii365·obd2.ltd)</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="22" t="inlineStr">
+      <c r="A52" s="23" t="inlineStr">
         <is>
           <t>- BMW XM G09: IYZBK1 키(X5·X6·X7·XM 공용, UWB) — G섀시 BDC3 키 복사·추가 대상(Xhorse G chassis BDC3)</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="22" t="inlineStr">
+      <c r="A53" s="23" t="inlineStr">
         <is>
           <t>- BMW X4 F26 2016: 순정 CAS4+ 키 칩은 PCF7953(ID49) — PCF7945P는 "CAS4 modified type" 애프터마켓 키 칩(mk3·vvdi)이라 뺌</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="22" t="inlineStr">
+      <c r="A54" s="23" t="inlineStr">
         <is>
           <t>- BMW E90 CAS3+: 순정 키 칩 PCF7945·PCF7943·PCF7944 모두 ID46(Hitag2) 계열로 병존(bimmerfest·keyecu) — 자료 상충 아님</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="22" t="inlineStr">
+      <c r="A55" s="23" t="inlineStr">
         <is>
           <t>- BMW X3 G45: Lonsdor K518 PRO "2025 BMW X3 UWB에 BCP 키 추가" 절차(U섀시 BCP) 확인 — 이모빌라이저 BCP 확정</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="22" t="inlineStr">
+      <c r="A56" s="23" t="inlineStr">
         <is>
           <t>- BMW X3 F25 2013: CAS4+ 순정 키 칩 PCF7953(ID49) — 같이 적혀 있던 PCF7945P는 중국산 CAS4 호환 키 칩(mr-key·tlkeys 판매품)이라 뺌(X4 F26과 같은 판단)</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="22" t="n"/>
+      <c r="A57" s="23" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="22" t="inlineStr">
+      <c r="A58" s="23" t="inlineStr">
         <is>
           <t>※ 행 구분 규칙</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="22" t="inlineStr">
+      <c r="A59" s="23" t="inlineStr">
         <is>
           <t>- 연식 중간에 칩·이모빌라이저·키가 바뀐 해는 바뀌기 전·후를 따로 행으로 나눔. 세대가 바뀌면 세대별 모델명으로 1행씩, 같은 세대 안의 변경(부분변경·생산 시기·키 변경)은 같은 모델명으로 나누고 칸 안의 [생산 시기]·[세대] 표기로 구분</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="22" t="inlineStr">
+      <c r="A60" s="23" t="inlineStr">
         <is>
           <t>- 같은 연식·모델에 행이 2개인데 칸에 시기 표기가 없으면(예: 벤츠 FBS3 행과 FBS4 행) 전환 시점 자료가 없는 것 — 주황색, 비고의 방법(VIN 등)으로 확인</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="22" t="inlineStr">
+      <c r="A61" s="23" t="inlineStr">
         <is>
           <t>- BMW 순정 부품번호(애프터마켓 대체): 비상키 51215A4FBE5 = F40·F44·G20·G22·G26·G42·G80·G82 등 인서트 키(recambiosyaccesoriosbmw), 51215A65D30 = U06·U10·U11·G60·G70·I20 등 인서트 키, 리모컨 66125A473F4(M 스포츠, ECE+RoW+US) = F40·F44·F9x·G01·G42·G87·G80·G82(hubauer·딜러몰), 66125A47402(기본, ECE+RoW) = G01·G02·G08·G11·G12·G30(schmiedmann), 66125A56076(기본, ECE+RoW) = F15·F16·F39·F45·F46·F48(hubauer), 66128708328(기본, ECE+RoW+US) = F40·G29(hubauer), 66125B3E8E1(M, ECE+RoW) = G60·G70·I20·U06·U10·U11 등, 66129362173 = i3 I01 434MHz(66126805980 대체), 51217127047 = X3 E83 도어·점화 키 — 한국 사양(KO) 번호 적용 차종은 미확인이라 [해외 공용 품번]</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="22" t="inlineStr">
-        <is>
-          <t>- BMW ETK(etkbmw.cc, 카탈로그 03.2019) 키 부품: 한국 사양(L802A National version Korea) 조건 번호가 있으면 그대로(태그 없음), 없으면 국가 제한 없는 번호를 [해외 공용 품번]으로 기재. 한국 사양 CAS 리모컨은 315MHz 저출력 전용 품번(예: 66126986584 = E60·E63·E70·E71·E84·E89 등, 2005.9 이전 E60·E63은 66126933076), E83 X3 한국 사양은 적외선 리모컨 51218374933도 등재. 트림 태그(기본형·스포츠 라인·럭셔리 라인·M 스포츠 등)는 ETK 키 디자인 구분, M 모델은 M·M 스포츠·디스플레이키·컴포트액세스만. 2021년식 이후와 E38·E39는 카탈로그 범위 밖이라 미기재</t>
+      <c r="A62" s="23" t="inlineStr">
+        <is>
+          <t>- BMW ETK(etkbmw.cc, 카탈로그 03.2019) 키 부품: 한국 사양(L802A National version Korea) 조건 번호가 있으면 그대로(태그 없음), 없으면 국가 제한 없는 번호를 [해외 공용 품번]으로 기재. 주파수: F·G·I 계열(2009년경~) 한국 사양 키는 434MHz(ETK 표기 434 MHZ KO·KOREA). 단 E 계열(CAS2·CAS3, 2003~2014년경 E60·E63·E65·E70·E71·E84·E89·E8x·1M)은 ETK에서 한국 사양(L802A 적용) 키가 315MHz 저출력(일본과 공용)으로만 등재되고 434MHz 키(예: 66126933075·66126986582)는 한국 사양 제외(L802A 미적용) 조건이라, 국내 사양 번호로 315MHz 저출력 품번을 기재(예: 66126986584, 2005.9 이전 E60·E63은 66126933076, 컴포트액세스 66126986580·66129268487, E65 66126959045). E83 X3 한국 사양은 적외선 리모컨 51218374933도 등재. 트림 태그(기본형·스포츠 라인·럭셔리 라인·M 스포츠 등)는 ETK 키 디자인 구분, M 모델은 M·M 스포츠·디스플레이키·컴포트액세스만. 2021년식 이후와 E38·E39는 카탈로그 범위 밖이라 미기재</t>
         </is>
       </c>
     </row>

</xml_diff>